<commit_message>
Excel lesson 1 (part 2): Lists sheet with named ranges lstStatus and lstPriority
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,20 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC77BEAF-2E51-D041-998B-D1E651C09672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB55E16-8F3E-F147-B6AB-B3A53A345A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
-    <sheet name="About" sheetId="2" r:id="rId2"/>
+    <sheet name="Lists" sheetId="3" r:id="rId2"/>
+    <sheet name="About" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="lstPriority">Lists!$B$2:$B$4</definedName>
+    <definedName name="lstStatus">Lists!$A$2:$A$5</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="237">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -3579,6 +3584,53 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F401B4-D906-1C43-878F-E6A45225E5F5}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Excel lesson 1 (part 3): dropdown validation for Status and Priority (J2:K61)
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB55E16-8F3E-F147-B6AB-B3A53A345A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A200182-311F-7E49-B616-4C8BB51A5663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
@@ -3576,6 +3576,14 @@
       <c r="M61" s="2"/>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J61" xr:uid="{1600F5D8-DEFE-FF4B-8562-B698D15E1FD4}">
+      <formula1>lstPriority</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K61" xr:uid="{426E204B-DEE8-544E-A485-F57F7D235EF0}">
+      <formula1>lstStatus</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Excel lesson 2 (part 1): add Suppliers lookup sheet (record ID -> golden record -> segment)
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A200182-311F-7E49-B616-4C8BB51A5663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FB188C-0FE0-6942-B30C-D03679BC384A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
     <sheet name="Lists" sheetId="3" r:id="rId2"/>
     <sheet name="About" sheetId="2" r:id="rId3"/>
+    <sheet name="Suppliers" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="lstPriority">Lists!$B$2:$B$4</definedName>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="557">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -737,6 +738,966 @@
   </si>
   <si>
     <t>Created date, status, owner and closed date are simulated for the Excel exercises. Owners are fictional.</t>
+  </si>
+  <si>
+    <t>Golden ID</t>
+  </si>
+  <si>
+    <t>Golden Name</t>
+  </si>
+  <si>
+    <t>Segment</t>
+  </si>
+  <si>
+    <t>G0001</t>
+  </si>
+  <si>
+    <t>Reliable, lower spend</t>
+  </si>
+  <si>
+    <t>0000100254</t>
+  </si>
+  <si>
+    <t>G0002</t>
+  </si>
+  <si>
+    <t>Ferroform s.r.o.</t>
+  </si>
+  <si>
+    <t>Critical: quality and delivery</t>
+  </si>
+  <si>
+    <t>SUP-0043</t>
+  </si>
+  <si>
+    <t>0000100075</t>
+  </si>
+  <si>
+    <t>G0003</t>
+  </si>
+  <si>
+    <t>Atlaswerk GmbH</t>
+  </si>
+  <si>
+    <t>Delivery risk</t>
+  </si>
+  <si>
+    <t>0000100099</t>
+  </si>
+  <si>
+    <t>G0004</t>
+  </si>
+  <si>
+    <t>Ventoline S.r.l.</t>
+  </si>
+  <si>
+    <t>SUP-0021</t>
+  </si>
+  <si>
+    <t>0000100048</t>
+  </si>
+  <si>
+    <t>G0005</t>
+  </si>
+  <si>
+    <t>Lumenflex SAS</t>
+  </si>
+  <si>
+    <t>0000100206</t>
+  </si>
+  <si>
+    <t>G0006</t>
+  </si>
+  <si>
+    <t>Aquametal GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0036</t>
+  </si>
+  <si>
+    <t>0000100046</t>
+  </si>
+  <si>
+    <t>G0007</t>
+  </si>
+  <si>
+    <t>Orbiscast s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100351</t>
+  </si>
+  <si>
+    <t>G0008</t>
+  </si>
+  <si>
+    <t>Polarparts GmbH</t>
+  </si>
+  <si>
+    <t>G0009</t>
+  </si>
+  <si>
+    <t>Strategic and reliable</t>
+  </si>
+  <si>
+    <t>0000100203</t>
+  </si>
+  <si>
+    <t>G0010</t>
+  </si>
+  <si>
+    <t>Deltaguss GmbH</t>
+  </si>
+  <si>
+    <t>0000100069</t>
+  </si>
+  <si>
+    <t>G0011</t>
+  </si>
+  <si>
+    <t>Cerrocast s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100169</t>
+  </si>
+  <si>
+    <t>G0012</t>
+  </si>
+  <si>
+    <t>Velawerk s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100084</t>
+  </si>
+  <si>
+    <t>G0013</t>
+  </si>
+  <si>
+    <t>Tauroparts S.r.l.</t>
+  </si>
+  <si>
+    <t>0000100271</t>
+  </si>
+  <si>
+    <t>G0014</t>
+  </si>
+  <si>
+    <t>Velaparts s.r.o.</t>
+  </si>
+  <si>
+    <t>Quality risk</t>
+  </si>
+  <si>
+    <t>0000100388</t>
+  </si>
+  <si>
+    <t>G0015</t>
+  </si>
+  <si>
+    <t>Silberline S.r.l.</t>
+  </si>
+  <si>
+    <t>G0016</t>
+  </si>
+  <si>
+    <t>0000100014</t>
+  </si>
+  <si>
+    <t>G0017</t>
+  </si>
+  <si>
+    <t>Novawerk GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0003</t>
+  </si>
+  <si>
+    <t>G0018</t>
+  </si>
+  <si>
+    <t>0000100027</t>
+  </si>
+  <si>
+    <t>G0019</t>
+  </si>
+  <si>
+    <t>Kraftguss s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100154</t>
+  </si>
+  <si>
+    <t>G0020</t>
+  </si>
+  <si>
+    <t>Boraseal GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0029</t>
+  </si>
+  <si>
+    <t>0000100115</t>
+  </si>
+  <si>
+    <t>G0021</t>
+  </si>
+  <si>
+    <t>Velaguss Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>SUP-0022</t>
+  </si>
+  <si>
+    <t>0000100142</t>
+  </si>
+  <si>
+    <t>G0022</t>
+  </si>
+  <si>
+    <t>Velacast GmbH</t>
+  </si>
+  <si>
+    <t>0000100230</t>
+  </si>
+  <si>
+    <t>G0023</t>
+  </si>
+  <si>
+    <t>Taurometal Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>0000100417</t>
+  </si>
+  <si>
+    <t>G0024</t>
+  </si>
+  <si>
+    <t>NORDCAST SP. Z O.O.</t>
+  </si>
+  <si>
+    <t>0000100136</t>
+  </si>
+  <si>
+    <t>G0025</t>
+  </si>
+  <si>
+    <t>0000100338</t>
+  </si>
+  <si>
+    <t>G0026</t>
+  </si>
+  <si>
+    <t>Kappaplast GmbH</t>
+  </si>
+  <si>
+    <t>0000100422</t>
+  </si>
+  <si>
+    <t>G0027</t>
+  </si>
+  <si>
+    <t>PRIMAFORM S.R.L.</t>
+  </si>
+  <si>
+    <t>SUP-0038</t>
+  </si>
+  <si>
+    <t>0000100261</t>
+  </si>
+  <si>
+    <t>G0028</t>
+  </si>
+  <si>
+    <t>Novaseal GmbH</t>
+  </si>
+  <si>
+    <t>0000100108</t>
+  </si>
+  <si>
+    <t>G0029</t>
+  </si>
+  <si>
+    <t>Ventoseal GmbH</t>
+  </si>
+  <si>
+    <t>0000100401</t>
+  </si>
+  <si>
+    <t>G0030</t>
+  </si>
+  <si>
+    <t>Silbermetal s.r.o.</t>
+  </si>
+  <si>
+    <t>SUP-0075</t>
+  </si>
+  <si>
+    <t>G0031</t>
+  </si>
+  <si>
+    <t>0000100386</t>
+  </si>
+  <si>
+    <t>G0032</t>
+  </si>
+  <si>
+    <t>Voltacast GmbH</t>
+  </si>
+  <si>
+    <t>0000100190</t>
+  </si>
+  <si>
+    <t>G0033</t>
+  </si>
+  <si>
+    <t>Primaplast S.r.l.</t>
+  </si>
+  <si>
+    <t>0000100311</t>
+  </si>
+  <si>
+    <t>G0034</t>
+  </si>
+  <si>
+    <t>Novametal Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>SUP-0059</t>
+  </si>
+  <si>
+    <t>G0035</t>
+  </si>
+  <si>
+    <t>SUP-0037</t>
+  </si>
+  <si>
+    <t>0000100412</t>
+  </si>
+  <si>
+    <t>G0036</t>
+  </si>
+  <si>
+    <t>Atlasguss  GmbH</t>
+  </si>
+  <si>
+    <t>0000100043</t>
+  </si>
+  <si>
+    <t>G0037</t>
+  </si>
+  <si>
+    <t>Ferroflex GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0011</t>
+  </si>
+  <si>
+    <t>0000100244</t>
+  </si>
+  <si>
+    <t>G0038</t>
+  </si>
+  <si>
+    <t>Voltawerk GmbH</t>
+  </si>
+  <si>
+    <t>G0039</t>
+  </si>
+  <si>
+    <t>0000100151</t>
+  </si>
+  <si>
+    <t>G0040</t>
+  </si>
+  <si>
+    <t>Nordguss SAS</t>
+  </si>
+  <si>
+    <t>G0041</t>
+  </si>
+  <si>
+    <t>G0042</t>
+  </si>
+  <si>
+    <t>G0043</t>
+  </si>
+  <si>
+    <t>0000100299</t>
+  </si>
+  <si>
+    <t>G0044</t>
+  </si>
+  <si>
+    <t>Ventoplast GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0052</t>
+  </si>
+  <si>
+    <t>G0045</t>
+  </si>
+  <si>
+    <t>0000100377</t>
+  </si>
+  <si>
+    <t>G0046</t>
+  </si>
+  <si>
+    <t>Nordline GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0073</t>
+  </si>
+  <si>
+    <t>G0047</t>
+  </si>
+  <si>
+    <t>G0048</t>
+  </si>
+  <si>
+    <t>0000100180</t>
+  </si>
+  <si>
+    <t>G0049</t>
+  </si>
+  <si>
+    <t>Novaline GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0033</t>
+  </si>
+  <si>
+    <t>0000100395</t>
+  </si>
+  <si>
+    <t>G0050</t>
+  </si>
+  <si>
+    <t>Atlasflex GmbH</t>
+  </si>
+  <si>
+    <t>G0051</t>
+  </si>
+  <si>
+    <t>0000100026</t>
+  </si>
+  <si>
+    <t>G0052</t>
+  </si>
+  <si>
+    <t>Krafttec GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0007</t>
+  </si>
+  <si>
+    <t>0000100192</t>
+  </si>
+  <si>
+    <t>G0053</t>
+  </si>
+  <si>
+    <t>Lumenform GmbH</t>
+  </si>
+  <si>
+    <t>0000100398</t>
+  </si>
+  <si>
+    <t>G0054</t>
+  </si>
+  <si>
+    <t>Terratronic GmbH</t>
+  </si>
+  <si>
+    <t>0000100040</t>
+  </si>
+  <si>
+    <t>G0055</t>
+  </si>
+  <si>
+    <t>Atlasform s.r.o.</t>
+  </si>
+  <si>
+    <t>SUP-0010</t>
+  </si>
+  <si>
+    <t>0000100325</t>
+  </si>
+  <si>
+    <t>G0056</t>
+  </si>
+  <si>
+    <t>Deltaform Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>0000100358</t>
+  </si>
+  <si>
+    <t>G0057</t>
+  </si>
+  <si>
+    <t>Ventotronic GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0070</t>
+  </si>
+  <si>
+    <t>G0058</t>
+  </si>
+  <si>
+    <t>0000100368</t>
+  </si>
+  <si>
+    <t>G0059</t>
+  </si>
+  <si>
+    <t>Alpencast Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>SUP-0072</t>
+  </si>
+  <si>
+    <t>0000100263</t>
+  </si>
+  <si>
+    <t>G0060</t>
+  </si>
+  <si>
+    <t>Atlasparts Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>0000100356</t>
+  </si>
+  <si>
+    <t>G0061</t>
+  </si>
+  <si>
+    <t>Kraftflex s.r.o.</t>
+  </si>
+  <si>
+    <t>G0062</t>
+  </si>
+  <si>
+    <t>0000100286</t>
+  </si>
+  <si>
+    <t>G0063</t>
+  </si>
+  <si>
+    <t>Polarcast Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>0000100320</t>
+  </si>
+  <si>
+    <t>G0064</t>
+  </si>
+  <si>
+    <t>Deltacast GmbH</t>
+  </si>
+  <si>
+    <t>0000100391</t>
+  </si>
+  <si>
+    <t>G0065</t>
+  </si>
+  <si>
+    <t>Kappaform GmbH</t>
+  </si>
+  <si>
+    <t>0000100310</t>
+  </si>
+  <si>
+    <t>G0066</t>
+  </si>
+  <si>
+    <t>0000100090</t>
+  </si>
+  <si>
+    <t>G0067</t>
+  </si>
+  <si>
+    <t>Polarmetal s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100029</t>
+  </si>
+  <si>
+    <t>G0068</t>
+  </si>
+  <si>
+    <t>Deltametal Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>0000100277</t>
+  </si>
+  <si>
+    <t>G0069</t>
+  </si>
+  <si>
+    <t>Lumenwerk s.r.o.</t>
+  </si>
+  <si>
+    <t>G0070</t>
+  </si>
+  <si>
+    <t>SUP-0002</t>
+  </si>
+  <si>
+    <t>G0071</t>
+  </si>
+  <si>
+    <t>G0072</t>
+  </si>
+  <si>
+    <t>0000100243</t>
+  </si>
+  <si>
+    <t>G0073</t>
+  </si>
+  <si>
+    <t>Ventoguss GmbH</t>
+  </si>
+  <si>
+    <t>0000100196</t>
+  </si>
+  <si>
+    <t>G0074</t>
+  </si>
+  <si>
+    <t>Alpenguss SAS</t>
+  </si>
+  <si>
+    <t>0000100035</t>
+  </si>
+  <si>
+    <t>G0075</t>
+  </si>
+  <si>
+    <t>Silberguss GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0009</t>
+  </si>
+  <si>
+    <t>0000100210</t>
+  </si>
+  <si>
+    <t>G0076</t>
+  </si>
+  <si>
+    <t>Aquatronic GmbH</t>
+  </si>
+  <si>
+    <t>0000100366</t>
+  </si>
+  <si>
+    <t>G0077</t>
+  </si>
+  <si>
+    <t>Orbisparts GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0071</t>
+  </si>
+  <si>
+    <t>0000100406</t>
+  </si>
+  <si>
+    <t>G0078</t>
+  </si>
+  <si>
+    <t>Velaseal s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100060</t>
+  </si>
+  <si>
+    <t>G0079</t>
+  </si>
+  <si>
+    <t>Primaparts GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0015</t>
+  </si>
+  <si>
+    <t>0000100292</t>
+  </si>
+  <si>
+    <t>G0080</t>
+  </si>
+  <si>
+    <t>Velaline S.r.l.</t>
+  </si>
+  <si>
+    <t>0000100120</t>
+  </si>
+  <si>
+    <t>G0081</t>
+  </si>
+  <si>
+    <t>Aquaplast s.r.o.</t>
+  </si>
+  <si>
+    <t>0000100405</t>
+  </si>
+  <si>
+    <t>G0082</t>
+  </si>
+  <si>
+    <t>Ferrotronic S.r.l.</t>
+  </si>
+  <si>
+    <t>0000100342</t>
+  </si>
+  <si>
+    <t>G0083</t>
+  </si>
+  <si>
+    <t>Kappawerk GmbH</t>
+  </si>
+  <si>
+    <t>G0084</t>
+  </si>
+  <si>
+    <t>0000100346</t>
+  </si>
+  <si>
+    <t>G0085</t>
+  </si>
+  <si>
+    <t>Voltatec GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0051</t>
+  </si>
+  <si>
+    <t>G0086</t>
+  </si>
+  <si>
+    <t>Terraseal  SAS</t>
+  </si>
+  <si>
+    <t>SUP-0014</t>
+  </si>
+  <si>
+    <t>G0087</t>
+  </si>
+  <si>
+    <t>Polarplast  S.r.l.</t>
+  </si>
+  <si>
+    <t>SUP-0013</t>
+  </si>
+  <si>
+    <t>G0088</t>
+  </si>
+  <si>
+    <t>Orbisguss</t>
+  </si>
+  <si>
+    <t>SUP-0053</t>
+  </si>
+  <si>
+    <t>G0089</t>
+  </si>
+  <si>
+    <t>Boratc S.r.l.</t>
+  </si>
+  <si>
+    <t>SUP-0028</t>
+  </si>
+  <si>
+    <t>G0090</t>
+  </si>
+  <si>
+    <t>Tauroseal</t>
+  </si>
+  <si>
+    <t>G0091</t>
+  </si>
+  <si>
+    <t>SUP-0046</t>
+  </si>
+  <si>
+    <t>G0092</t>
+  </si>
+  <si>
+    <t>RHEINSEAL GMBH</t>
+  </si>
+  <si>
+    <t>SUP-0031</t>
+  </si>
+  <si>
+    <t>G0093</t>
+  </si>
+  <si>
+    <t>Orbistronic</t>
+  </si>
+  <si>
+    <t>G0094</t>
+  </si>
+  <si>
+    <t>SUP-0067</t>
+  </si>
+  <si>
+    <t>G0095</t>
+  </si>
+  <si>
+    <t>Cerrotec GmbH</t>
+  </si>
+  <si>
+    <t>G0096</t>
+  </si>
+  <si>
+    <t>G0097</t>
+  </si>
+  <si>
+    <t>SUP-0017</t>
+  </si>
+  <si>
+    <t>G0098</t>
+  </si>
+  <si>
+    <t>KAPPATEC GMBH</t>
+  </si>
+  <si>
+    <t>SUP-0050</t>
+  </si>
+  <si>
+    <t>G0099</t>
+  </si>
+  <si>
+    <t>Boraflex  s.r.o.</t>
+  </si>
+  <si>
+    <t>G0100</t>
+  </si>
+  <si>
+    <t>SUP-0066</t>
+  </si>
+  <si>
+    <t>G0101</t>
+  </si>
+  <si>
+    <t>RHEINGUSS SAS</t>
+  </si>
+  <si>
+    <t>SUP-0004</t>
+  </si>
+  <si>
+    <t>G0102</t>
+  </si>
+  <si>
+    <t>Deltaarts SAS</t>
+  </si>
+  <si>
+    <t>SUP-0063</t>
+  </si>
+  <si>
+    <t>G0103</t>
+  </si>
+  <si>
+    <t>TAUROGUSS GMBH</t>
+  </si>
+  <si>
+    <t>SUP-0064</t>
+  </si>
+  <si>
+    <t>G0104</t>
+  </si>
+  <si>
+    <t>VELAFORM GMBH</t>
+  </si>
+  <si>
+    <t>G0105</t>
+  </si>
+  <si>
+    <t>SUP-0035</t>
+  </si>
+  <si>
+    <t>G0106</t>
+  </si>
+  <si>
+    <t>Veltec GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0062</t>
+  </si>
+  <si>
+    <t>G0107</t>
+  </si>
+  <si>
+    <t>Nordtronic</t>
+  </si>
+  <si>
+    <t>G0108</t>
+  </si>
+  <si>
+    <t>G0109</t>
+  </si>
+  <si>
+    <t>G0110</t>
+  </si>
+  <si>
+    <t>G0111</t>
+  </si>
+  <si>
+    <t>G0112</t>
+  </si>
+  <si>
+    <t>G0113</t>
+  </si>
+  <si>
+    <t>SUP-0045</t>
+  </si>
+  <si>
+    <t>G0114</t>
+  </si>
+  <si>
+    <t>Orbisflex GmbH</t>
+  </si>
+  <si>
+    <t>SUP-0049</t>
+  </si>
+  <si>
+    <t>G0115</t>
+  </si>
+  <si>
+    <t>Deltatc s.r.o.</t>
+  </si>
+  <si>
+    <t>G0116</t>
+  </si>
+  <si>
+    <t>G0117</t>
+  </si>
+  <si>
+    <t>SUP-0068</t>
+  </si>
+  <si>
+    <t>G0118</t>
+  </si>
+  <si>
+    <t>Cerroform  S.r.l.</t>
+  </si>
+  <si>
+    <t>SUP-0026</t>
+  </si>
+  <si>
+    <t>G0119</t>
+  </si>
+  <si>
+    <t>Voltasal Sp. z o.o.</t>
+  </si>
+  <si>
+    <t>SUP-0048</t>
+  </si>
+  <si>
+    <t>G0120</t>
+  </si>
+  <si>
+    <t>Taurotec  GmbH</t>
   </si>
 </sst>
 </file>
@@ -781,15 +1742,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -808,12 +1776,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -828,11 +1790,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:M61" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:M61" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:M61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -843,7 +1805,7 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3661,4 +4623,2826 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{693EEE6C-E3E0-E544-A038-BEFFA0B97036}">
+  <dimension ref="A1:E165"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D4" t="s">
+        <v>244</v>
+      </c>
+      <c r="E4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="s">
+        <v>248</v>
+      </c>
+      <c r="D5" t="s">
+        <v>249</v>
+      </c>
+      <c r="E5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
+        <v>252</v>
+      </c>
+      <c r="D7" t="s">
+        <v>253</v>
+      </c>
+      <c r="E7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" t="s">
+        <v>253</v>
+      </c>
+      <c r="E8" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D9" t="s">
+        <v>257</v>
+      </c>
+      <c r="E9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
+        <v>259</v>
+      </c>
+      <c r="D10" t="s">
+        <v>260</v>
+      </c>
+      <c r="E10" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>259</v>
+      </c>
+      <c r="D11" t="s">
+        <v>260</v>
+      </c>
+      <c r="E11" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>263</v>
+      </c>
+      <c r="D12" t="s">
+        <v>264</v>
+      </c>
+      <c r="E12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" t="s">
+        <v>266</v>
+      </c>
+      <c r="D13" t="s">
+        <v>267</v>
+      </c>
+      <c r="E13" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" t="s">
+        <v>268</v>
+      </c>
+      <c r="D14" t="s">
+        <v>117</v>
+      </c>
+      <c r="E14" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" t="s">
+        <v>271</v>
+      </c>
+      <c r="D15" t="s">
+        <v>272</v>
+      </c>
+      <c r="E15" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" t="s">
+        <v>274</v>
+      </c>
+      <c r="D16" t="s">
+        <v>275</v>
+      </c>
+      <c r="E16" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>274</v>
+      </c>
+      <c r="D17" t="s">
+        <v>275</v>
+      </c>
+      <c r="E17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" t="s">
+        <v>277</v>
+      </c>
+      <c r="D18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E18" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
+        <v>277</v>
+      </c>
+      <c r="D19" t="s">
+        <v>278</v>
+      </c>
+      <c r="E19" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" t="s">
+        <v>280</v>
+      </c>
+      <c r="D20" t="s">
+        <v>281</v>
+      </c>
+      <c r="E20" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" t="s">
+        <v>283</v>
+      </c>
+      <c r="D21" t="s">
+        <v>284</v>
+      </c>
+      <c r="E21" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B22" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" t="s">
+        <v>287</v>
+      </c>
+      <c r="D22" t="s">
+        <v>288</v>
+      </c>
+      <c r="E22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" t="s">
+        <v>289</v>
+      </c>
+      <c r="D23" t="s">
+        <v>123</v>
+      </c>
+      <c r="E23" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D24" t="s">
+        <v>292</v>
+      </c>
+      <c r="E24" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" t="s">
+        <v>291</v>
+      </c>
+      <c r="D25" t="s">
+        <v>292</v>
+      </c>
+      <c r="E25" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" t="s">
+        <v>294</v>
+      </c>
+      <c r="D26" t="s">
+        <v>129</v>
+      </c>
+      <c r="E26" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" t="s">
+        <v>296</v>
+      </c>
+      <c r="D27" t="s">
+        <v>297</v>
+      </c>
+      <c r="E27" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" t="s">
+        <v>296</v>
+      </c>
+      <c r="D28" t="s">
+        <v>297</v>
+      </c>
+      <c r="E28" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
+        <v>299</v>
+      </c>
+      <c r="D29" t="s">
+        <v>300</v>
+      </c>
+      <c r="E29" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>299</v>
+      </c>
+      <c r="D30" t="s">
+        <v>300</v>
+      </c>
+      <c r="E30" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="B31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" t="s">
+        <v>303</v>
+      </c>
+      <c r="D31" t="s">
+        <v>304</v>
+      </c>
+      <c r="E31" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B32" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" t="s">
+        <v>303</v>
+      </c>
+      <c r="D32" t="s">
+        <v>304</v>
+      </c>
+      <c r="E32" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="B33" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" t="s">
+        <v>307</v>
+      </c>
+      <c r="D33" t="s">
+        <v>308</v>
+      </c>
+      <c r="E33" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" t="s">
+        <v>307</v>
+      </c>
+      <c r="D34" t="s">
+        <v>308</v>
+      </c>
+      <c r="E34" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="B35" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" t="s">
+        <v>310</v>
+      </c>
+      <c r="D35" t="s">
+        <v>311</v>
+      </c>
+      <c r="E35" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B36" t="s">
+        <v>108</v>
+      </c>
+      <c r="C36" t="s">
+        <v>313</v>
+      </c>
+      <c r="D36" t="s">
+        <v>314</v>
+      </c>
+      <c r="E36" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B37" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" t="s">
+        <v>313</v>
+      </c>
+      <c r="D37" t="s">
+        <v>314</v>
+      </c>
+      <c r="E37" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B38" t="s">
+        <v>108</v>
+      </c>
+      <c r="C38" t="s">
+        <v>316</v>
+      </c>
+      <c r="D38" t="s">
+        <v>188</v>
+      </c>
+      <c r="E38" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" t="s">
+        <v>316</v>
+      </c>
+      <c r="D39" t="s">
+        <v>188</v>
+      </c>
+      <c r="E39" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" t="s">
+        <v>318</v>
+      </c>
+      <c r="D40" t="s">
+        <v>319</v>
+      </c>
+      <c r="E40" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" t="s">
+        <v>318</v>
+      </c>
+      <c r="D41" t="s">
+        <v>319</v>
+      </c>
+      <c r="E41" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B42" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" t="s">
+        <v>321</v>
+      </c>
+      <c r="D42" t="s">
+        <v>322</v>
+      </c>
+      <c r="E42" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B43" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" t="s">
+        <v>321</v>
+      </c>
+      <c r="D43" t="s">
+        <v>322</v>
+      </c>
+      <c r="E43" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" t="s">
+        <v>321</v>
+      </c>
+      <c r="D44" t="s">
+        <v>322</v>
+      </c>
+      <c r="E44" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="B45" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" t="s">
+        <v>325</v>
+      </c>
+      <c r="D45" t="s">
+        <v>326</v>
+      </c>
+      <c r="E45" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" t="s">
+        <v>325</v>
+      </c>
+      <c r="D46" t="s">
+        <v>326</v>
+      </c>
+      <c r="E46" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B47" t="s">
+        <v>108</v>
+      </c>
+      <c r="C47" t="s">
+        <v>328</v>
+      </c>
+      <c r="D47" t="s">
+        <v>329</v>
+      </c>
+      <c r="E47" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B48" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" t="s">
+        <v>331</v>
+      </c>
+      <c r="D48" t="s">
+        <v>332</v>
+      </c>
+      <c r="E48" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="B49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" t="s">
+        <v>331</v>
+      </c>
+      <c r="D49" t="s">
+        <v>332</v>
+      </c>
+      <c r="E49" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B50" t="s">
+        <v>108</v>
+      </c>
+      <c r="C50" t="s">
+        <v>334</v>
+      </c>
+      <c r="D50" t="s">
+        <v>132</v>
+      </c>
+      <c r="E50" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B51" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" t="s">
+        <v>336</v>
+      </c>
+      <c r="D51" t="s">
+        <v>337</v>
+      </c>
+      <c r="E51" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" t="s">
+        <v>339</v>
+      </c>
+      <c r="D52" t="s">
+        <v>340</v>
+      </c>
+      <c r="E52" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" t="s">
+        <v>339</v>
+      </c>
+      <c r="D53" t="s">
+        <v>340</v>
+      </c>
+      <c r="E53" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B54" t="s">
+        <v>108</v>
+      </c>
+      <c r="C54" t="s">
+        <v>342</v>
+      </c>
+      <c r="D54" t="s">
+        <v>343</v>
+      </c>
+      <c r="E54" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B55" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" t="s">
+        <v>342</v>
+      </c>
+      <c r="D55" t="s">
+        <v>343</v>
+      </c>
+      <c r="E55" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B56" t="s">
+        <v>108</v>
+      </c>
+      <c r="C56" t="s">
+        <v>345</v>
+      </c>
+      <c r="D56" t="s">
+        <v>135</v>
+      </c>
+      <c r="E56" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="B57" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" t="s">
+        <v>345</v>
+      </c>
+      <c r="D57" t="s">
+        <v>135</v>
+      </c>
+      <c r="E57" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="B58" t="s">
+        <v>108</v>
+      </c>
+      <c r="C58" t="s">
+        <v>348</v>
+      </c>
+      <c r="D58" t="s">
+        <v>349</v>
+      </c>
+      <c r="E58" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B59" t="s">
+        <v>108</v>
+      </c>
+      <c r="C59" t="s">
+        <v>348</v>
+      </c>
+      <c r="D59" t="s">
+        <v>349</v>
+      </c>
+      <c r="E59" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B60" t="s">
+        <v>108</v>
+      </c>
+      <c r="C60" t="s">
+        <v>351</v>
+      </c>
+      <c r="D60" t="s">
+        <v>352</v>
+      </c>
+      <c r="E60" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="B61" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" t="s">
+        <v>351</v>
+      </c>
+      <c r="D61" t="s">
+        <v>352</v>
+      </c>
+      <c r="E61" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="B62" t="s">
+        <v>108</v>
+      </c>
+      <c r="C62" t="s">
+        <v>355</v>
+      </c>
+      <c r="D62" t="s">
+        <v>356</v>
+      </c>
+      <c r="E62" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B63" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" t="s">
+        <v>355</v>
+      </c>
+      <c r="D63" t="s">
+        <v>356</v>
+      </c>
+      <c r="E63" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B64" t="s">
+        <v>108</v>
+      </c>
+      <c r="C64" t="s">
+        <v>357</v>
+      </c>
+      <c r="D64" t="s">
+        <v>138</v>
+      </c>
+      <c r="E64" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="B65" t="s">
+        <v>108</v>
+      </c>
+      <c r="C65" t="s">
+        <v>359</v>
+      </c>
+      <c r="D65" t="s">
+        <v>360</v>
+      </c>
+      <c r="E65" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B66" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66" t="s">
+        <v>359</v>
+      </c>
+      <c r="D66" t="s">
+        <v>360</v>
+      </c>
+      <c r="E66" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B67" t="s">
+        <v>108</v>
+      </c>
+      <c r="C67" t="s">
+        <v>361</v>
+      </c>
+      <c r="D67" t="s">
+        <v>144</v>
+      </c>
+      <c r="E67" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B68" t="s">
+        <v>108</v>
+      </c>
+      <c r="C68" t="s">
+        <v>362</v>
+      </c>
+      <c r="D68" t="s">
+        <v>148</v>
+      </c>
+      <c r="E68" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B69" t="s">
+        <v>108</v>
+      </c>
+      <c r="C69" t="s">
+        <v>363</v>
+      </c>
+      <c r="D69" t="s">
+        <v>152</v>
+      </c>
+      <c r="E69" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="B70" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" t="s">
+        <v>365</v>
+      </c>
+      <c r="D70" t="s">
+        <v>366</v>
+      </c>
+      <c r="E70" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="B71" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" t="s">
+        <v>365</v>
+      </c>
+      <c r="D71" t="s">
+        <v>366</v>
+      </c>
+      <c r="E71" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B72" t="s">
+        <v>108</v>
+      </c>
+      <c r="C72" t="s">
+        <v>368</v>
+      </c>
+      <c r="D72" t="s">
+        <v>155</v>
+      </c>
+      <c r="E72" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="B73" t="s">
+        <v>108</v>
+      </c>
+      <c r="C73" t="s">
+        <v>370</v>
+      </c>
+      <c r="D73" t="s">
+        <v>371</v>
+      </c>
+      <c r="E73" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="B74" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74" t="s">
+        <v>370</v>
+      </c>
+      <c r="D74" t="s">
+        <v>371</v>
+      </c>
+      <c r="E74" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B75" t="s">
+        <v>108</v>
+      </c>
+      <c r="C75" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" t="s">
+        <v>160</v>
+      </c>
+      <c r="E75" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B76" t="s">
+        <v>108</v>
+      </c>
+      <c r="C76" t="s">
+        <v>374</v>
+      </c>
+      <c r="D76" t="s">
+        <v>163</v>
+      </c>
+      <c r="E76" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B77" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" t="s">
+        <v>374</v>
+      </c>
+      <c r="D77" t="s">
+        <v>163</v>
+      </c>
+      <c r="E77" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B78" t="s">
+        <v>108</v>
+      </c>
+      <c r="C78" t="s">
+        <v>376</v>
+      </c>
+      <c r="D78" t="s">
+        <v>377</v>
+      </c>
+      <c r="E78" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" t="s">
+        <v>377</v>
+      </c>
+      <c r="E79" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="B80" t="s">
+        <v>108</v>
+      </c>
+      <c r="C80" t="s">
+        <v>380</v>
+      </c>
+      <c r="D80" t="s">
+        <v>381</v>
+      </c>
+      <c r="E80" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B81" t="s">
+        <v>108</v>
+      </c>
+      <c r="C81" t="s">
+        <v>382</v>
+      </c>
+      <c r="D81" t="s">
+        <v>166</v>
+      </c>
+      <c r="E81" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="B82" t="s">
+        <v>108</v>
+      </c>
+      <c r="C82" t="s">
+        <v>384</v>
+      </c>
+      <c r="D82" t="s">
+        <v>385</v>
+      </c>
+      <c r="E82" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="B83" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" t="s">
+        <v>385</v>
+      </c>
+      <c r="E83" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B84" t="s">
+        <v>108</v>
+      </c>
+      <c r="C84" t="s">
+        <v>388</v>
+      </c>
+      <c r="D84" t="s">
+        <v>389</v>
+      </c>
+      <c r="E84" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B85" t="s">
+        <v>108</v>
+      </c>
+      <c r="C85" t="s">
+        <v>388</v>
+      </c>
+      <c r="D85" t="s">
+        <v>389</v>
+      </c>
+      <c r="E85" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B86" t="s">
+        <v>108</v>
+      </c>
+      <c r="C86" t="s">
+        <v>391</v>
+      </c>
+      <c r="D86" t="s">
+        <v>392</v>
+      </c>
+      <c r="E86" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B87" t="s">
+        <v>108</v>
+      </c>
+      <c r="C87" t="s">
+        <v>394</v>
+      </c>
+      <c r="D87" t="s">
+        <v>395</v>
+      </c>
+      <c r="E87" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="B88" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" t="s">
+        <v>394</v>
+      </c>
+      <c r="D88" t="s">
+        <v>395</v>
+      </c>
+      <c r="E88" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="B89" t="s">
+        <v>108</v>
+      </c>
+      <c r="C89" t="s">
+        <v>398</v>
+      </c>
+      <c r="D89" t="s">
+        <v>399</v>
+      </c>
+      <c r="E89" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B90" t="s">
+        <v>108</v>
+      </c>
+      <c r="C90" t="s">
+        <v>401</v>
+      </c>
+      <c r="D90" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="B91" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91" t="s">
+        <v>401</v>
+      </c>
+      <c r="D91" t="s">
+        <v>402</v>
+      </c>
+      <c r="E91" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B92" t="s">
+        <v>108</v>
+      </c>
+      <c r="C92" t="s">
+        <v>404</v>
+      </c>
+      <c r="D92" t="s">
+        <v>169</v>
+      </c>
+      <c r="E92" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B93" t="s">
+        <v>14</v>
+      </c>
+      <c r="C93" t="s">
+        <v>404</v>
+      </c>
+      <c r="D93" t="s">
+        <v>169</v>
+      </c>
+      <c r="E93" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="B94" t="s">
+        <v>108</v>
+      </c>
+      <c r="C94" t="s">
+        <v>406</v>
+      </c>
+      <c r="D94" t="s">
+        <v>407</v>
+      </c>
+      <c r="E94" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="B95" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95" t="s">
+        <v>406</v>
+      </c>
+      <c r="D95" t="s">
+        <v>407</v>
+      </c>
+      <c r="E95" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="B96" t="s">
+        <v>108</v>
+      </c>
+      <c r="C96" t="s">
+        <v>410</v>
+      </c>
+      <c r="D96" t="s">
+        <v>411</v>
+      </c>
+      <c r="E96" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="B97" t="s">
+        <v>108</v>
+      </c>
+      <c r="C97" t="s">
+        <v>413</v>
+      </c>
+      <c r="D97" t="s">
+        <v>414</v>
+      </c>
+      <c r="E97" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B98" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" t="s">
+        <v>413</v>
+      </c>
+      <c r="D98" t="s">
+        <v>414</v>
+      </c>
+      <c r="E98" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A99" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B99" t="s">
+        <v>108</v>
+      </c>
+      <c r="C99" t="s">
+        <v>415</v>
+      </c>
+      <c r="D99" t="s">
+        <v>172</v>
+      </c>
+      <c r="E99" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="B100" t="s">
+        <v>108</v>
+      </c>
+      <c r="C100" t="s">
+        <v>417</v>
+      </c>
+      <c r="D100" t="s">
+        <v>418</v>
+      </c>
+      <c r="E100" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="B101" t="s">
+        <v>108</v>
+      </c>
+      <c r="C101" t="s">
+        <v>420</v>
+      </c>
+      <c r="D101" t="s">
+        <v>421</v>
+      </c>
+      <c r="E101" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="B102" t="s">
+        <v>108</v>
+      </c>
+      <c r="C102" t="s">
+        <v>423</v>
+      </c>
+      <c r="D102" t="s">
+        <v>424</v>
+      </c>
+      <c r="E102" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="B103" t="s">
+        <v>108</v>
+      </c>
+      <c r="C103" t="s">
+        <v>426</v>
+      </c>
+      <c r="D103" t="s">
+        <v>26</v>
+      </c>
+      <c r="E103" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A104" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B104" t="s">
+        <v>14</v>
+      </c>
+      <c r="C104" t="s">
+        <v>426</v>
+      </c>
+      <c r="D104" t="s">
+        <v>26</v>
+      </c>
+      <c r="E104" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="B105" t="s">
+        <v>108</v>
+      </c>
+      <c r="C105" t="s">
+        <v>428</v>
+      </c>
+      <c r="D105" t="s">
+        <v>429</v>
+      </c>
+      <c r="E105" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B106" t="s">
+        <v>14</v>
+      </c>
+      <c r="C106" t="s">
+        <v>428</v>
+      </c>
+      <c r="D106" t="s">
+        <v>429</v>
+      </c>
+      <c r="E106" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B107" t="s">
+        <v>108</v>
+      </c>
+      <c r="C107" t="s">
+        <v>431</v>
+      </c>
+      <c r="D107" t="s">
+        <v>432</v>
+      </c>
+      <c r="E107" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B108" t="s">
+        <v>108</v>
+      </c>
+      <c r="C108" t="s">
+        <v>434</v>
+      </c>
+      <c r="D108" t="s">
+        <v>435</v>
+      </c>
+      <c r="E108" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B109" t="s">
+        <v>14</v>
+      </c>
+      <c r="C109" t="s">
+        <v>434</v>
+      </c>
+      <c r="D109" t="s">
+        <v>435</v>
+      </c>
+      <c r="E109" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B110" t="s">
+        <v>108</v>
+      </c>
+      <c r="C110" t="s">
+        <v>436</v>
+      </c>
+      <c r="D110" t="s">
+        <v>175</v>
+      </c>
+      <c r="E110" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B111" t="s">
+        <v>14</v>
+      </c>
+      <c r="C111" t="s">
+        <v>436</v>
+      </c>
+      <c r="D111" t="s">
+        <v>175</v>
+      </c>
+      <c r="E111" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B112" t="s">
+        <v>108</v>
+      </c>
+      <c r="C112" t="s">
+        <v>438</v>
+      </c>
+      <c r="D112" t="s">
+        <v>178</v>
+      </c>
+      <c r="E112" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B113" t="s">
+        <v>108</v>
+      </c>
+      <c r="C113" t="s">
+        <v>439</v>
+      </c>
+      <c r="D113" t="s">
+        <v>181</v>
+      </c>
+      <c r="E113" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A114" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B114" t="s">
+        <v>108</v>
+      </c>
+      <c r="C114" t="s">
+        <v>441</v>
+      </c>
+      <c r="D114" t="s">
+        <v>442</v>
+      </c>
+      <c r="E114" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B115" t="s">
+        <v>14</v>
+      </c>
+      <c r="C115" t="s">
+        <v>441</v>
+      </c>
+      <c r="D115" t="s">
+        <v>442</v>
+      </c>
+      <c r="E115" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="B116" t="s">
+        <v>108</v>
+      </c>
+      <c r="C116" t="s">
+        <v>444</v>
+      </c>
+      <c r="D116" t="s">
+        <v>445</v>
+      </c>
+      <c r="E116" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B117" t="s">
+        <v>108</v>
+      </c>
+      <c r="C117" t="s">
+        <v>447</v>
+      </c>
+      <c r="D117" t="s">
+        <v>448</v>
+      </c>
+      <c r="E117" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A118" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="B118" t="s">
+        <v>14</v>
+      </c>
+      <c r="C118" t="s">
+        <v>447</v>
+      </c>
+      <c r="D118" t="s">
+        <v>448</v>
+      </c>
+      <c r="E118" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B119" t="s">
+        <v>108</v>
+      </c>
+      <c r="C119" t="s">
+        <v>451</v>
+      </c>
+      <c r="D119" t="s">
+        <v>452</v>
+      </c>
+      <c r="E119" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A120" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="B120" t="s">
+        <v>108</v>
+      </c>
+      <c r="C120" t="s">
+        <v>454</v>
+      </c>
+      <c r="D120" t="s">
+        <v>455</v>
+      </c>
+      <c r="E120" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A121" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="B121" t="s">
+        <v>14</v>
+      </c>
+      <c r="C121" t="s">
+        <v>454</v>
+      </c>
+      <c r="D121" t="s">
+        <v>455</v>
+      </c>
+      <c r="E121" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A122" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="B122" t="s">
+        <v>108</v>
+      </c>
+      <c r="C122" t="s">
+        <v>458</v>
+      </c>
+      <c r="D122" t="s">
+        <v>459</v>
+      </c>
+      <c r="E122" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A123" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B123" t="s">
+        <v>108</v>
+      </c>
+      <c r="C123" t="s">
+        <v>461</v>
+      </c>
+      <c r="D123" t="s">
+        <v>462</v>
+      </c>
+      <c r="E123" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="B124" t="s">
+        <v>14</v>
+      </c>
+      <c r="C124" t="s">
+        <v>461</v>
+      </c>
+      <c r="D124" t="s">
+        <v>462</v>
+      </c>
+      <c r="E124" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B125" t="s">
+        <v>108</v>
+      </c>
+      <c r="C125" t="s">
+        <v>465</v>
+      </c>
+      <c r="D125" t="s">
+        <v>466</v>
+      </c>
+      <c r="E125" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="B126" t="s">
+        <v>108</v>
+      </c>
+      <c r="C126" t="s">
+        <v>468</v>
+      </c>
+      <c r="D126" t="s">
+        <v>469</v>
+      </c>
+      <c r="E126" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="B127" t="s">
+        <v>108</v>
+      </c>
+      <c r="C127" t="s">
+        <v>471</v>
+      </c>
+      <c r="D127" t="s">
+        <v>472</v>
+      </c>
+      <c r="E127" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A128" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B128" t="s">
+        <v>108</v>
+      </c>
+      <c r="C128" t="s">
+        <v>474</v>
+      </c>
+      <c r="D128" t="s">
+        <v>475</v>
+      </c>
+      <c r="E128" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A129" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B129" t="s">
+        <v>108</v>
+      </c>
+      <c r="C129" t="s">
+        <v>476</v>
+      </c>
+      <c r="D129" t="s">
+        <v>185</v>
+      </c>
+      <c r="E129" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B130" t="s">
+        <v>108</v>
+      </c>
+      <c r="C130" t="s">
+        <v>478</v>
+      </c>
+      <c r="D130" t="s">
+        <v>479</v>
+      </c>
+      <c r="E130" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A131" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B131" t="s">
+        <v>14</v>
+      </c>
+      <c r="C131" t="s">
+        <v>481</v>
+      </c>
+      <c r="D131" t="s">
+        <v>482</v>
+      </c>
+      <c r="E131" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A132" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="B132" t="s">
+        <v>14</v>
+      </c>
+      <c r="C132" t="s">
+        <v>484</v>
+      </c>
+      <c r="D132" t="s">
+        <v>485</v>
+      </c>
+      <c r="E132" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A133" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B133" t="s">
+        <v>14</v>
+      </c>
+      <c r="C133" t="s">
+        <v>487</v>
+      </c>
+      <c r="D133" t="s">
+        <v>488</v>
+      </c>
+      <c r="E133" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A134" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="B134" t="s">
+        <v>14</v>
+      </c>
+      <c r="C134" t="s">
+        <v>490</v>
+      </c>
+      <c r="D134" t="s">
+        <v>491</v>
+      </c>
+      <c r="E134" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A135" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B135" t="s">
+        <v>14</v>
+      </c>
+      <c r="C135" t="s">
+        <v>493</v>
+      </c>
+      <c r="D135" t="s">
+        <v>494</v>
+      </c>
+      <c r="E135" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A136" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B136" t="s">
+        <v>14</v>
+      </c>
+      <c r="C136" t="s">
+        <v>495</v>
+      </c>
+      <c r="D136" t="s">
+        <v>51</v>
+      </c>
+      <c r="E136" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A137" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B137" t="s">
+        <v>14</v>
+      </c>
+      <c r="C137" t="s">
+        <v>497</v>
+      </c>
+      <c r="D137" t="s">
+        <v>498</v>
+      </c>
+      <c r="E137" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A138" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="B138" t="s">
+        <v>14</v>
+      </c>
+      <c r="C138" t="s">
+        <v>500</v>
+      </c>
+      <c r="D138" t="s">
+        <v>501</v>
+      </c>
+      <c r="E138" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A139" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B139" t="s">
+        <v>14</v>
+      </c>
+      <c r="C139" t="s">
+        <v>502</v>
+      </c>
+      <c r="D139" t="s">
+        <v>197</v>
+      </c>
+      <c r="E139" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A140" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B140" t="s">
+        <v>14</v>
+      </c>
+      <c r="C140" t="s">
+        <v>504</v>
+      </c>
+      <c r="D140" t="s">
+        <v>505</v>
+      </c>
+      <c r="E140" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A141" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B141" t="s">
+        <v>14</v>
+      </c>
+      <c r="C141" t="s">
+        <v>506</v>
+      </c>
+      <c r="D141" t="s">
+        <v>206</v>
+      </c>
+      <c r="E141" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A142" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B142" t="s">
+        <v>14</v>
+      </c>
+      <c r="C142" t="s">
+        <v>507</v>
+      </c>
+      <c r="D142" t="s">
+        <v>209</v>
+      </c>
+      <c r="E142" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A143" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="B143" t="s">
+        <v>14</v>
+      </c>
+      <c r="C143" t="s">
+        <v>509</v>
+      </c>
+      <c r="D143" t="s">
+        <v>510</v>
+      </c>
+      <c r="E143" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A144" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B144" t="s">
+        <v>14</v>
+      </c>
+      <c r="C144" t="s">
+        <v>512</v>
+      </c>
+      <c r="D144" t="s">
+        <v>513</v>
+      </c>
+      <c r="E144" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A145" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B145" t="s">
+        <v>14</v>
+      </c>
+      <c r="C145" t="s">
+        <v>514</v>
+      </c>
+      <c r="D145" t="s">
+        <v>63</v>
+      </c>
+      <c r="E145" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A146" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B146" t="s">
+        <v>14</v>
+      </c>
+      <c r="C146" t="s">
+        <v>516</v>
+      </c>
+      <c r="D146" t="s">
+        <v>517</v>
+      </c>
+      <c r="E146" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A147" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="B147" t="s">
+        <v>14</v>
+      </c>
+      <c r="C147" t="s">
+        <v>519</v>
+      </c>
+      <c r="D147" t="s">
+        <v>520</v>
+      </c>
+      <c r="E147" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A148" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="B148" t="s">
+        <v>14</v>
+      </c>
+      <c r="C148" t="s">
+        <v>522</v>
+      </c>
+      <c r="D148" t="s">
+        <v>523</v>
+      </c>
+      <c r="E148" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A149" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="B149" t="s">
+        <v>14</v>
+      </c>
+      <c r="C149" t="s">
+        <v>525</v>
+      </c>
+      <c r="D149" t="s">
+        <v>526</v>
+      </c>
+      <c r="E149" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A150" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B150" t="s">
+        <v>14</v>
+      </c>
+      <c r="C150" t="s">
+        <v>527</v>
+      </c>
+      <c r="D150" t="s">
+        <v>66</v>
+      </c>
+      <c r="E150" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A151" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="B151" t="s">
+        <v>14</v>
+      </c>
+      <c r="C151" t="s">
+        <v>529</v>
+      </c>
+      <c r="D151" t="s">
+        <v>530</v>
+      </c>
+      <c r="E151" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A152" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="B152" t="s">
+        <v>14</v>
+      </c>
+      <c r="C152" t="s">
+        <v>532</v>
+      </c>
+      <c r="D152" t="s">
+        <v>533</v>
+      </c>
+      <c r="E152" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A153" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B153" t="s">
+        <v>14</v>
+      </c>
+      <c r="C153" t="s">
+        <v>534</v>
+      </c>
+      <c r="D153" t="s">
+        <v>69</v>
+      </c>
+      <c r="E153" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A154" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B154" t="s">
+        <v>14</v>
+      </c>
+      <c r="C154" t="s">
+        <v>535</v>
+      </c>
+      <c r="D154" t="s">
+        <v>72</v>
+      </c>
+      <c r="E154" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A155" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B155" t="s">
+        <v>14</v>
+      </c>
+      <c r="C155" t="s">
+        <v>536</v>
+      </c>
+      <c r="D155" t="s">
+        <v>76</v>
+      </c>
+      <c r="E155" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A156" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B156" t="s">
+        <v>14</v>
+      </c>
+      <c r="C156" t="s">
+        <v>537</v>
+      </c>
+      <c r="D156" t="s">
+        <v>79</v>
+      </c>
+      <c r="E156" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A157" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B157" t="s">
+        <v>14</v>
+      </c>
+      <c r="C157" t="s">
+        <v>538</v>
+      </c>
+      <c r="D157" t="s">
+        <v>82</v>
+      </c>
+      <c r="E157" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A158" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B158" t="s">
+        <v>14</v>
+      </c>
+      <c r="C158" t="s">
+        <v>539</v>
+      </c>
+      <c r="D158" t="s">
+        <v>85</v>
+      </c>
+      <c r="E158" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A159" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="B159" t="s">
+        <v>14</v>
+      </c>
+      <c r="C159" t="s">
+        <v>541</v>
+      </c>
+      <c r="D159" t="s">
+        <v>542</v>
+      </c>
+      <c r="E159" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A160" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B160" t="s">
+        <v>14</v>
+      </c>
+      <c r="C160" t="s">
+        <v>544</v>
+      </c>
+      <c r="D160" t="s">
+        <v>545</v>
+      </c>
+      <c r="E160" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A161" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B161" t="s">
+        <v>14</v>
+      </c>
+      <c r="C161" t="s">
+        <v>546</v>
+      </c>
+      <c r="D161" t="s">
+        <v>94</v>
+      </c>
+      <c r="E161" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A162" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B162" t="s">
+        <v>14</v>
+      </c>
+      <c r="C162" t="s">
+        <v>547</v>
+      </c>
+      <c r="D162" t="s">
+        <v>100</v>
+      </c>
+      <c r="E162" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A163" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="B163" t="s">
+        <v>14</v>
+      </c>
+      <c r="C163" t="s">
+        <v>549</v>
+      </c>
+      <c r="D163" t="s">
+        <v>550</v>
+      </c>
+      <c r="E163" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A164" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B164" t="s">
+        <v>14</v>
+      </c>
+      <c r="C164" t="s">
+        <v>552</v>
+      </c>
+      <c r="D164" t="s">
+        <v>553</v>
+      </c>
+      <c r="E164" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A165" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="B165" t="s">
+        <v>14</v>
+      </c>
+      <c r="C165" t="s">
+        <v>555</v>
+      </c>
+      <c r="D165" t="s">
+        <v>556</v>
+      </c>
+      <c r="E165" t="s">
+        <v>269</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel lesson 2 (part 2): Segment column with XLOOKUP from Suppliers sheet
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FB188C-0FE0-6942-B30C-D03679BC384A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25982A9-BE03-3044-AF58-3E6564A69FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,25 @@
     <definedName name="lstPriority">Lists!$B$2:$B$4</definedName>
     <definedName name="lstStatus">Lists!$A$2:$A$5</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="557">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1751,7 +1764,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     </dxf>
@@ -1790,11 +1806,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:M61" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:M61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:N61" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:N61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1805,7 +1821,10 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2096,7 +2115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.1640625" customWidth="1"/>
@@ -2114,7 +2133,7 @@
     <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2154,8 +2173,14 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2195,8 +2220,12 @@
       <c r="M2" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N2" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2236,8 +2265,12 @@
       <c r="M3" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N3" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2275,8 +2308,12 @@
         <v>32</v>
       </c>
       <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N4" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2314,8 +2351,12 @@
         <v>41</v>
       </c>
       <c r="M5" s="2"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N5" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -2353,8 +2394,12 @@
         <v>45</v>
       </c>
       <c r="M6" s="2"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N6" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2394,8 +2439,12 @@
       <c r="M7" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -2435,8 +2484,12 @@
       <c r="M8" s="2">
         <v>46268</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N8" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -2474,8 +2527,12 @@
         <v>27</v>
       </c>
       <c r="M9" s="2"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N9" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -2515,8 +2572,12 @@
       <c r="M10" s="2">
         <v>46273</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N10" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2554,8 +2615,12 @@
         <v>41</v>
       </c>
       <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N11" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -2593,8 +2658,12 @@
         <v>45</v>
       </c>
       <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N12" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -2634,8 +2703,12 @@
       <c r="M13" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N13" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -2675,8 +2748,12 @@
       <c r="M14" s="2">
         <v>46277</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N14" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -2714,8 +2791,12 @@
         <v>45</v>
       </c>
       <c r="M15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N15" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -2753,8 +2834,12 @@
         <v>41</v>
       </c>
       <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N16" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2792,8 +2877,12 @@
         <v>45</v>
       </c>
       <c r="M17" s="2"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N17" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -2831,8 +2920,12 @@
         <v>45</v>
       </c>
       <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N18" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -2870,8 +2963,12 @@
         <v>23</v>
       </c>
       <c r="M19" s="2"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N19" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>86</v>
       </c>
@@ -2909,8 +3006,12 @@
         <v>27</v>
       </c>
       <c r="M20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N20" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>89</v>
       </c>
@@ -2948,8 +3049,12 @@
         <v>41</v>
       </c>
       <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N21" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>92</v>
       </c>
@@ -2987,8 +3092,12 @@
         <v>23</v>
       </c>
       <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N22" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>95</v>
       </c>
@@ -3026,8 +3135,12 @@
         <v>45</v>
       </c>
       <c r="M23" s="2"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N23" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>98</v>
       </c>
@@ -3065,8 +3178,12 @@
         <v>23</v>
       </c>
       <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N24" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>101</v>
       </c>
@@ -3106,8 +3223,12 @@
       <c r="M25" s="2">
         <v>46281</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N25" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -3145,8 +3266,12 @@
         <v>27</v>
       </c>
       <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N26" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>107</v>
       </c>
@@ -3186,8 +3311,12 @@
       <c r="M27" s="2">
         <v>46294</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N27" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -3227,8 +3356,12 @@
       <c r="M28" s="2">
         <v>46293</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N28" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -3268,8 +3401,12 @@
       <c r="M29" s="2">
         <v>46286</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N29" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>126</v>
       </c>
@@ -3307,8 +3444,12 @@
         <v>32</v>
       </c>
       <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N30" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -3346,8 +3487,12 @@
         <v>27</v>
       </c>
       <c r="M31" s="2"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N31" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>130</v>
       </c>
@@ -3385,8 +3530,12 @@
         <v>45</v>
       </c>
       <c r="M32" s="2"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N32" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>133</v>
       </c>
@@ -3426,8 +3575,12 @@
       <c r="M33" s="2">
         <v>46294</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N33" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>136</v>
       </c>
@@ -3465,8 +3618,12 @@
         <v>32</v>
       </c>
       <c r="M34" s="2"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N34" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>142</v>
       </c>
@@ -3504,8 +3661,12 @@
         <v>41</v>
       </c>
       <c r="M35" s="2"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N35" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>146</v>
       </c>
@@ -3543,8 +3704,12 @@
         <v>27</v>
       </c>
       <c r="M36" s="2"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N36" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>150</v>
       </c>
@@ -3584,8 +3749,12 @@
       <c r="M37" s="2">
         <v>46299</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N37" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>153</v>
       </c>
@@ -3623,8 +3792,12 @@
         <v>41</v>
       </c>
       <c r="M38" s="2"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N38" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>158</v>
       </c>
@@ -3664,8 +3837,12 @@
       <c r="M39" s="2">
         <v>46284</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N39" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -3705,8 +3882,12 @@
       <c r="M40" s="2">
         <v>46285</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N40" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>164</v>
       </c>
@@ -3746,8 +3927,12 @@
       <c r="M41" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N41" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>167</v>
       </c>
@@ -3785,8 +3970,12 @@
         <v>45</v>
       </c>
       <c r="M42" s="2"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N42" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>170</v>
       </c>
@@ -3824,8 +4013,12 @@
         <v>41</v>
       </c>
       <c r="M43" s="2"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N43" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>173</v>
       </c>
@@ -3865,8 +4058,12 @@
       <c r="M44" s="2">
         <v>46288</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N44" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>176</v>
       </c>
@@ -3906,8 +4103,12 @@
       <c r="M45" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N45" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -3945,8 +4146,12 @@
         <v>45</v>
       </c>
       <c r="M46" s="2"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N46" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>183</v>
       </c>
@@ -3984,8 +4189,12 @@
         <v>32</v>
       </c>
       <c r="M47" s="2"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N47" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>186</v>
       </c>
@@ -4023,8 +4232,12 @@
         <v>27</v>
       </c>
       <c r="M48" s="2"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N48" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>189</v>
       </c>
@@ -4062,8 +4275,12 @@
         <v>23</v>
       </c>
       <c r="M49" s="2"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N49" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>190</v>
       </c>
@@ -4101,8 +4318,12 @@
         <v>45</v>
       </c>
       <c r="M50" s="2"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N50" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -4140,8 +4361,12 @@
         <v>32</v>
       </c>
       <c r="M51" s="2"/>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N51" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -4179,8 +4404,12 @@
         <v>27</v>
       </c>
       <c r="M52" s="2"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N52" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>201</v>
       </c>
@@ -4220,8 +4449,12 @@
       <c r="M53" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N53" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>204</v>
       </c>
@@ -4259,8 +4492,12 @@
         <v>45</v>
       </c>
       <c r="M54" s="2"/>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N54" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>207</v>
       </c>
@@ -4300,8 +4537,12 @@
       <c r="M55" s="2">
         <v>46300</v>
       </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N55" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>211</v>
       </c>
@@ -4339,8 +4580,12 @@
         <v>45</v>
       </c>
       <c r="M56" s="2"/>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N56" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>212</v>
       </c>
@@ -4378,8 +4623,12 @@
         <v>41</v>
       </c>
       <c r="M57" s="2"/>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N57" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Quality risk</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>215</v>
       </c>
@@ -4417,8 +4666,12 @@
         <v>45</v>
       </c>
       <c r="M58" s="2"/>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N58" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Critical: quality and delivery</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>222</v>
       </c>
@@ -4456,8 +4709,12 @@
         <v>41</v>
       </c>
       <c r="M59" s="2"/>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N59" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Strategic and reliable</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>226</v>
       </c>
@@ -4497,8 +4754,12 @@
       <c r="M60" s="2">
         <v>46271</v>
       </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N60" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Reliable, lower spend</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>230</v>
       </c>
@@ -4536,6 +4797,10 @@
         <v>23</v>
       </c>
       <c r="M61" s="2"/>
+      <c r="N61" t="str">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
+        <v>Delivery risk</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Excel lesson 2 (part 3): Age (days) column with IF and TODAY; wider Segment column
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25982A9-BE03-3044-AF58-3E6564A69FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AB2291-F174-9641-ABA6-B13DD32C0AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="559">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1711,6 +1711,12 @@
   </si>
   <si>
     <t>Taurotec  GmbH</t>
+  </si>
+  <si>
+    <t>delivery risk</t>
+  </si>
+  <si>
+    <t>Age (days)</t>
   </si>
 </sst>
 </file>
@@ -1764,7 +1770,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1806,11 +1815,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:N61" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:N61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:O61" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:O61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1821,9 +1830,12 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="1"/>
-    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="0">
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="delivery risk" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="0">
+      <calculatedColumnFormula>IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2131,6 +2143,7 @@
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -2174,10 +2187,10 @@
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>239</v>
+        <v>557</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>239</v>
+        <v>558</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -2224,6 +2237,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O2">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>6</v>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -2268,6 +2285,10 @@
       <c r="N3" t="str">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
+      </c>
+      <c r="O3">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2312,6 +2333,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O4">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -2355,6 +2380,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O5">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>23</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -2398,6 +2427,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O6">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>25</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -2443,6 +2476,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
+      <c r="O7">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -2487,6 +2524,10 @@
       <c r="N8" t="str">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
+      </c>
+      <c r="O8">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2531,6 +2572,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
+      <c r="O9">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>32</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -2575,6 +2620,10 @@
       <c r="N10" t="str">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
+      </c>
+      <c r="O10">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2619,6 +2668,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
+      <c r="O11">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>22</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -2662,6 +2715,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O12">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -2707,6 +2764,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
+      <c r="O13">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>5</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -2751,6 +2812,10 @@
       <c r="N14" t="str">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
+      </c>
+      <c r="O14">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -2795,6 +2860,10 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
+      <c r="O15">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -2838,8 +2907,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O16">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2881,8 +2954,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O17">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -2924,8 +3001,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O18">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -2967,8 +3048,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O19">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>86</v>
       </c>
@@ -3010,8 +3095,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O20">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>89</v>
       </c>
@@ -3053,8 +3142,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O21">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>92</v>
       </c>
@@ -3096,8 +3189,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O22">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>95</v>
       </c>
@@ -3139,8 +3236,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O23">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>98</v>
       </c>
@@ -3182,8 +3283,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O24">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>101</v>
       </c>
@@ -3227,8 +3332,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O25">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -3270,8 +3379,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O26">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>107</v>
       </c>
@@ -3315,8 +3428,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O27">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -3360,8 +3477,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O28">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -3405,8 +3526,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O29">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>126</v>
       </c>
@@ -3448,8 +3573,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O30">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -3491,8 +3620,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O31">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>130</v>
       </c>
@@ -3534,8 +3667,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O32">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>133</v>
       </c>
@@ -3579,8 +3716,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O33">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>136</v>
       </c>
@@ -3622,8 +3763,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O34">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>142</v>
       </c>
@@ -3665,8 +3810,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O35">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>146</v>
       </c>
@@ -3708,8 +3857,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O36">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>150</v>
       </c>
@@ -3753,8 +3906,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O37">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>153</v>
       </c>
@@ -3796,8 +3953,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O38">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>158</v>
       </c>
@@ -3841,8 +4002,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O39">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -3886,8 +4051,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O40">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>164</v>
       </c>
@@ -3931,8 +4100,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O41">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>167</v>
       </c>
@@ -3974,8 +4147,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O42">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>170</v>
       </c>
@@ -4017,8 +4194,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O43">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>173</v>
       </c>
@@ -4062,8 +4243,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O44">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>176</v>
       </c>
@@ -4107,8 +4292,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O45">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -4150,8 +4339,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O46">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>183</v>
       </c>
@@ -4193,8 +4386,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O47">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>186</v>
       </c>
@@ -4236,8 +4433,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O48">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>189</v>
       </c>
@@ -4279,8 +4480,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O49">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>190</v>
       </c>
@@ -4322,8 +4527,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O50">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -4365,8 +4574,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O51">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -4408,8 +4621,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O52">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>201</v>
       </c>
@@ -4453,8 +4670,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O53">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>204</v>
       </c>
@@ -4496,8 +4717,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O54">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>207</v>
       </c>
@@ -4541,8 +4766,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O55">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>211</v>
       </c>
@@ -4584,8 +4813,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O56">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>212</v>
       </c>
@@ -4627,8 +4860,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Quality risk</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O57">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>215</v>
       </c>
@@ -4670,8 +4907,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Critical: quality and delivery</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O58">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>222</v>
       </c>
@@ -4713,8 +4954,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Strategic and reliable</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O59">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>226</v>
       </c>
@@ -4758,8 +5003,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Reliable, lower spend</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O60">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>230</v>
       </c>
@@ -4800,6 +5049,10 @@
       <c r="N61" t="str">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</f>
         <v>Delivery risk</v>
+      </c>
+      <c r="O61">
+        <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel lesson 2 (part 4): SLA targets in Lists sheet and SLA (days) column with XLOOKUP
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AB2291-F174-9641-ABA6-B13DD32C0AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FDF598-5B8F-FF43-AE59-F58248EC3F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="559">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1713,10 +1713,10 @@
     <t>Taurotec  GmbH</t>
   </si>
   <si>
-    <t>delivery risk</t>
-  </si>
-  <si>
     <t>Age (days)</t>
+  </si>
+  <si>
+    <t>SLA (days)</t>
   </si>
 </sst>
 </file>
@@ -1770,7 +1770,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1815,11 +1818,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:O61" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:O61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:P61" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:P61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1830,12 +1833,15 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="delivery risk" dataDxfId="1">
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="0">
+    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="1">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2127,7 +2133,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.1640625" customWidth="1"/>
@@ -2146,7 +2152,7 @@
     <col min="14" max="14" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2187,13 +2193,16 @@
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2241,8 +2250,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P2">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2290,8 +2303,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P3">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2337,8 +2354,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P4">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2384,8 +2405,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P5">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -2431,8 +2456,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P6">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2480,8 +2509,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P7">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -2529,8 +2562,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P8">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -2576,8 +2613,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P9">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -2625,8 +2666,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P10">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2672,8 +2717,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P11">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -2719,8 +2768,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P12">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -2768,8 +2821,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P13">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -2817,8 +2874,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P14">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -2864,8 +2925,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P15">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -2911,8 +2976,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P16">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2958,8 +3027,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P17">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -3005,8 +3078,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>34</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P18">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -3052,8 +3129,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P19">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>86</v>
       </c>
@@ -3099,8 +3180,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P20">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>89</v>
       </c>
@@ -3146,8 +3231,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>17</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P21">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>92</v>
       </c>
@@ -3193,8 +3282,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>13</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P22">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>95</v>
       </c>
@@ -3240,8 +3333,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>27</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P23">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>98</v>
       </c>
@@ -3287,8 +3384,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>34</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P24">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>101</v>
       </c>
@@ -3336,8 +3437,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P25">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -3383,8 +3488,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P26">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>107</v>
       </c>
@@ -3432,8 +3541,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P27">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -3481,8 +3594,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P28">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -3530,8 +3647,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P29">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>126</v>
       </c>
@@ -3577,8 +3698,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>23</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P30">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -3624,8 +3749,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>28</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P31">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>130</v>
       </c>
@@ -3671,8 +3800,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P32">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>133</v>
       </c>
@@ -3720,8 +3853,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>7</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P33">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>136</v>
       </c>
@@ -3767,8 +3904,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P34">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>142</v>
       </c>
@@ -3814,8 +3955,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P35">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>146</v>
       </c>
@@ -3861,8 +4006,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>11</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P36">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>150</v>
       </c>
@@ -3910,8 +4059,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P37">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>153</v>
       </c>
@@ -3957,8 +4110,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>23</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P38">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>158</v>
       </c>
@@ -4006,8 +4163,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P39">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -4055,8 +4216,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P40">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>164</v>
       </c>
@@ -4104,8 +4269,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P41">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>167</v>
       </c>
@@ -4151,8 +4320,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>8</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P42">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>170</v>
       </c>
@@ -4198,8 +4371,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>32</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P43">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>173</v>
       </c>
@@ -4247,8 +4424,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>7</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P44">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>176</v>
       </c>
@@ -4296,8 +4477,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P45">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -4343,8 +4528,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>16</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P46">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>183</v>
       </c>
@@ -4390,8 +4579,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P47">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>186</v>
       </c>
@@ -4437,8 +4630,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P48">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>189</v>
       </c>
@@ -4484,8 +4681,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>33</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P49">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>190</v>
       </c>
@@ -4531,8 +4732,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P50">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -4578,8 +4783,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>23</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P51">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -4625,8 +4834,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P52">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>201</v>
       </c>
@@ -4674,8 +4887,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P53">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>204</v>
       </c>
@@ -4721,8 +4938,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P54">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>207</v>
       </c>
@@ -4770,8 +4991,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P55">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>211</v>
       </c>
@@ -4817,8 +5042,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>33</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P56">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>212</v>
       </c>
@@ -4864,8 +5093,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P57">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>215</v>
       </c>
@@ -4911,8 +5144,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>14</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P58">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>222</v>
       </c>
@@ -4958,8 +5195,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P59">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>226</v>
       </c>
@@ -5007,8 +5248,12 @@
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P60">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>230</v>
       </c>
@@ -5053,6 +5298,10 @@
       <c r="O61">
         <f ca="1">IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</f>
         <v>12</v>
+      </c>
+      <c r="P61">
+        <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5073,42 +5322,54 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F401B4-D906-1C43-878F-E6A45225E5F5}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>40</v>
       </c>
       <c r="B2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>31</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>149</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Excel lesson 2 (part 5): SLA Status column (Breached/OK) with IF
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FDF598-5B8F-FF43-AE59-F58248EC3F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9825A41C-7966-2040-AD84-327C389B36D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="560">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1717,6 +1717,9 @@
   </si>
   <si>
     <t>SLA (days)</t>
+  </si>
+  <si>
+    <t>SLA Status</t>
   </si>
 </sst>
 </file>
@@ -1761,16 +1764,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1818,11 +1825,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:P61" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:P61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:Q61" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A1:Q61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
+  <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1833,15 +1840,18 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="2">
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="3">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="1">
+    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="2">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="0">
+    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{AD8149A7-3507-6C4D-829C-AB97FE40A20A}" name="SLA Status" dataDxfId="0">
+      <calculatedColumnFormula>IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2133,7 +2143,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.1640625" customWidth="1"/>
@@ -2150,9 +2160,10 @@
     <col min="12" max="12" width="11" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="28.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,8 +2212,11 @@
       <c r="P1" s="1" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="1" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2254,8 +2268,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2307,8 +2325,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q3" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2358,8 +2380,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q4" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2409,8 +2435,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q5" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -2460,8 +2490,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q6" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2513,8 +2547,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q7" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -2566,8 +2604,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q8" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -2617,8 +2659,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q9" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -2670,8 +2716,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q10" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2721,8 +2771,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q11" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -2772,8 +2826,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q12" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -2825,8 +2883,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q13" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -2878,8 +2940,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q14" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -2929,8 +2995,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q15" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -2980,8 +3050,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q16" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -3031,8 +3105,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q17" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -3082,8 +3160,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q18" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -3133,8 +3215,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q19" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>86</v>
       </c>
@@ -3184,8 +3270,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q20" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>89</v>
       </c>
@@ -3235,8 +3325,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q21" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>92</v>
       </c>
@@ -3286,8 +3380,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q22" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>95</v>
       </c>
@@ -3337,8 +3435,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q23" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>98</v>
       </c>
@@ -3388,8 +3490,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q24" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>101</v>
       </c>
@@ -3441,8 +3547,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q25" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -3492,8 +3602,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q26" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>107</v>
       </c>
@@ -3545,8 +3659,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q27" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -3598,8 +3716,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q28" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -3651,8 +3773,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q29" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>126</v>
       </c>
@@ -3702,8 +3828,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q30" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -3753,8 +3883,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q31" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>130</v>
       </c>
@@ -3804,8 +3938,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q32" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>133</v>
       </c>
@@ -3857,8 +3995,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q33" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>136</v>
       </c>
@@ -3908,8 +4050,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q34" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>142</v>
       </c>
@@ -3959,8 +4105,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q35" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>146</v>
       </c>
@@ -4010,8 +4160,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q36" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>150</v>
       </c>
@@ -4063,8 +4217,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q37" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>153</v>
       </c>
@@ -4114,8 +4272,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q38" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>158</v>
       </c>
@@ -4167,8 +4329,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q39" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -4220,8 +4386,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q40" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>164</v>
       </c>
@@ -4273,8 +4443,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q41" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>167</v>
       </c>
@@ -4324,8 +4498,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q42" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>170</v>
       </c>
@@ -4375,8 +4553,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q43" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>173</v>
       </c>
@@ -4428,8 +4610,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q44" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>176</v>
       </c>
@@ -4481,8 +4667,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q45" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -4532,8 +4722,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q46" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>183</v>
       </c>
@@ -4583,8 +4777,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q47" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>186</v>
       </c>
@@ -4634,8 +4832,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q48" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>189</v>
       </c>
@@ -4685,8 +4887,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q49" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>190</v>
       </c>
@@ -4736,8 +4942,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q50" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -4787,8 +4997,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q51" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -4838,8 +5052,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q52" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>201</v>
       </c>
@@ -4891,8 +5109,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q53" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>204</v>
       </c>
@@ -4942,8 +5164,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q54" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>207</v>
       </c>
@@ -4995,8 +5221,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q55" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>211</v>
       </c>
@@ -5046,8 +5276,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q56" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>212</v>
       </c>
@@ -5097,8 +5331,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q57" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>215</v>
       </c>
@@ -5148,8 +5386,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q58" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>222</v>
       </c>
@@ -5199,8 +5441,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q59" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>226</v>
       </c>
@@ -5252,8 +5498,12 @@
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q60" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>230</v>
       </c>
@@ -5302,6 +5552,10 @@
       <c r="P61">
         <f>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</f>
         <v>5</v>
+      </c>
+      <c r="Q61" s="4" t="str">
+        <f ca="1">IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</f>
+        <v>Breached</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel lesson 3 (part 1): Dashboard sheet with COUNTA, COUNTIF and COUNTIFS KPIs
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9825A41C-7966-2040-AD84-327C389B36D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9143E38-D634-FF43-8C73-657A1CC8FC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tickets" sheetId="1" r:id="rId1"/>
-    <sheet name="Lists" sheetId="3" r:id="rId2"/>
-    <sheet name="About" sheetId="2" r:id="rId3"/>
-    <sheet name="Suppliers" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" r:id="rId1"/>
+    <sheet name="Tickets" sheetId="1" r:id="rId2"/>
+    <sheet name="Lists" sheetId="3" r:id="rId3"/>
+    <sheet name="About" sheetId="2" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="lstPriority">Lists!$B$2:$B$4</definedName>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="564">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1720,6 +1721,18 @@
   </si>
   <si>
     <t>SLA Status</t>
+  </si>
+  <si>
+    <t>BU2 Ticket Dashboard</t>
+  </si>
+  <si>
+    <t>Total tickets</t>
+  </si>
+  <si>
+    <t>Open tickets</t>
+  </si>
+  <si>
+    <t>Open &amp; SLA breached</t>
   </si>
 </sst>
 </file>
@@ -2142,6 +2155,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12509E95-5F09-DC49-B9BC-77DD19A10A22}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>561</v>
+      </c>
+      <c r="B3">
+        <f>COUNTA(tblTickets[Ticket ID])</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(tblTickets[Status],"&lt;&gt;Closed")</f>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>563</v>
+      </c>
+      <c r="B5">
+        <f ca="1">COUNTIFS(tblTickets[Status],"&lt;&gt;Closed",tblTickets[SLA Status],"Breached")</f>
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -5574,7 +5632,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F401B4-D906-1C43-878F-E6A45225E5F5}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -5633,7 +5691,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -5658,7 +5716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{693EEE6C-E3E0-E544-A038-BEFFA0B97036}">
   <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Excel lesson 3 (part 2): conditional formatting highlights SLA breaches
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9143E38-D634-FF43-8C73-657A1CC8FC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B5C5C7-DFA8-9A4E-A449-A539510B7DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="5" r:id="rId1"/>
@@ -1787,7 +1787,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1838,11 +1848,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:Q61" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:Q61" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="A1:Q61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1853,17 +1863,17 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="4"/>
-    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="3">
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="2">
+    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="3">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="1">
+    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{AD8149A7-3507-6C4D-829C-AB97FE40A20A}" name="SLA Status" dataDxfId="0">
+    <tableColumn id="17" xr3:uid="{AD8149A7-3507-6C4D-829C-AB97FE40A20A}" name="SLA Status" dataDxfId="1">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5617,6 +5627,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="Q2:Q61">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Breached">
+      <formula>NOT(ISERROR(SEARCH("Breached",Q2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J61" xr:uid="{1600F5D8-DEFE-FF4B-8562-B698D15E1FD4}">
       <formula1>lstPriority</formula1>

</xml_diff>

<commit_message>
Excel lesson 3 (part 3): neutral table style so SLA breaches stand out
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B5C5C7-DFA8-9A4E-A449-A539510B7DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC202A7F-62A9-7843-B1F9-00DDEC1E48A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1787,7 +1787,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1848,11 +1868,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:Q61" totalsRowShown="0" headerRowDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}" name="tblTickets" displayName="tblTickets" ref="A1:Q61" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A1:Q61" xr:uid="{CA4F919C-D01A-DA41-A42E-110E3B4395C0}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{BE142A8F-F154-1044-B387-8577F406E53F}" name="Ticket ID"/>
-    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{D3303C1F-3E66-9847-9F7D-1BAB0A591DCB}" name="Created On" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{B7D3D6B8-C9F8-CB4E-A562-D40AB4479284}" name="System"/>
     <tableColumn id="4" xr3:uid="{F93E4226-D363-744D-9393-FC55010FB293}" name="Record ID"/>
     <tableColumn id="5" xr3:uid="{C5533319-CAEC-484D-B517-4DCE538BB5CF}" name="Supplier"/>
@@ -1863,21 +1883,21 @@
     <tableColumn id="10" xr3:uid="{38379D94-F847-8649-86DA-658C708DFA9F}" name="Priority"/>
     <tableColumn id="11" xr3:uid="{30BB1311-A968-9E47-9109-6B108A47B1AF}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FE767F43-C074-0E48-9423-F4F2AA52E313}" name="Owner"/>
-    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="4">
+    <tableColumn id="13" xr3:uid="{B0911052-D2D4-564C-9789-A5F9984A3638}" name="Closed On" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{5E7D163A-759D-984D-A1ED-C1B920E4AFE3}" name="Segment" dataDxfId="6">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Record ID]],Suppliers!A:A,Suppliers!E:E,"Not found")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="3">
+    <tableColumn id="15" xr3:uid="{7A46C142-8722-F24D-90F5-98A7C1A349EE}" name="Age (days)" dataDxfId="5">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Closed On]]="",TODAY()-tblTickets[[#This Row],[Created On]],tblTickets[[#This Row],[Closed On]]-tblTickets[[#This Row],[Created On]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="2">
+    <tableColumn id="16" xr3:uid="{4846F765-EDED-4B44-9C2B-4A17E4417593}" name="SLA (days)" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblTickets[[#This Row],[Priority]],Lists!B:B,Lists!C:C)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{AD8149A7-3507-6C4D-829C-AB97FE40A20A}" name="SLA Status" dataDxfId="1">
+    <tableColumn id="17" xr3:uid="{AD8149A7-3507-6C4D-829C-AB97FE40A20A}" name="SLA Status" dataDxfId="3">
       <calculatedColumnFormula>IF(tblTickets[[#This Row],[Age (days)]]&gt;tblTickets[[#This Row],[SLA (days)]],"Breached","OK")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -5628,7 +5648,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="Q2:Q61">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Breached">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Breached">
+      <formula>NOT(ISERROR(SEARCH("Breached",Q2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Breached">
       <formula>NOT(ISERROR(SEARCH("Breached",Q2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Excel lesson 3 (part 4): PivotTable on Dashboard - tickets by supplier segment and SLA status
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC202A7F-62A9-7843-B1F9-00DDEC1E48A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE441EC-A384-0D46-A1BB-2EFD8476A3F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="5" r:id="rId1"/>
@@ -24,6 +24,9 @@
     <definedName name="lstStatus">Lists!$A$2:$A$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId6"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="570">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -1733,6 +1736,24 @@
   </si>
   <si>
     <t>Open &amp; SLA breached</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Breached</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Count of Ticket ID</t>
   </si>
 </sst>
 </file>
@@ -1777,12 +1798,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1865,6 +1890,1315 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="mac" refreshedDate="46300.604069444445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="60" xr:uid="{E198A4B9-9466-014B-B142-729ED828A4DF}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="tblTickets"/>
+  </cacheSource>
+  <cacheFields count="17">
+    <cacheField name="Ticket ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Created On" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-09-01T00:00:00" maxDate="2026-10-04T00:00:00"/>
+    </cacheField>
+    <cacheField name="System" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Record ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Supplier" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Field" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="DQ Dimension" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Issue" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Suggested Action" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Priority" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Status" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Owner" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Closed On" numFmtId="164">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-09-03T00:00:00" maxDate="2026-10-06T00:00:00"/>
+    </cacheField>
+    <cacheField name="Segment" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Critical: quality and delivery"/>
+        <s v="Strategic and reliable"/>
+        <s v="Delivery risk"/>
+        <s v="Reliable, lower spend"/>
+        <s v="Quality risk"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Age (days)" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="34"/>
+    </cacheField>
+    <cacheField name="SLA (days)" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="5" maxValue="20"/>
+    </cacheField>
+    <cacheField name="SLA Status" numFmtId="0">
+      <sharedItems count="2">
+        <s v="OK"/>
+        <s v="Breached"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="60">
+  <r>
+    <s v="T-0001"/>
+    <d v="2026-09-29T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0065"/>
+    <s v="Kappaplast"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="0"/>
+    <n v="6"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0002"/>
+    <d v="2026-10-03T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0057"/>
+    <s v="Boratronic SAS"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="1"/>
+    <n v="2"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0003"/>
+    <d v="2026-10-03T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0047"/>
+    <s v="LUMENWERK S.R.O."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="In Progress"/>
+    <s v="J. Novak"/>
+    <m/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0004"/>
+    <d v="2026-09-12T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0042"/>
+    <s v="Voltawerk"/>
+    <s v="country"/>
+    <s v="consistency"/>
+    <s v="Country is not a standard English name / ISO code"/>
+    <s v="Map to ISO code DE"/>
+    <s v="Medium"/>
+    <s v="Open"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="0"/>
+    <n v="23"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0005"/>
+    <d v="2026-09-10T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0016"/>
+    <s v="CERROCAST S.R.O."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="25"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0006"/>
+    <d v="2026-09-26T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0018"/>
+    <s v="Atlaswerk"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="2"/>
+    <n v="9"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0007"/>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0019"/>
+    <s v="Nordplast  s.r.o."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="A. Weber"/>
+    <d v="2026-09-03T00:00:00"/>
+    <x v="2"/>
+    <n v="2"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0008"/>
+    <d v="2026-09-03T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0027"/>
+    <s v="Nordguss"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="3"/>
+    <n v="32"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0009"/>
+    <d v="2026-09-02T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0034"/>
+    <s v="Primaplast"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-09-08T00:00:00"/>
+    <x v="4"/>
+    <n v="6"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0010"/>
+    <d v="2026-09-13T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0032"/>
+    <s v="Velawek s.r.o."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="In Progress"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="1"/>
+    <n v="22"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0011"/>
+    <d v="2026-10-02T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0055"/>
+    <s v="Aquaparts  GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="3"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0012"/>
+    <d v="2026-09-30T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0074"/>
+    <s v="Silbercast  GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="J. Novak"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="3"/>
+    <n v="5"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0013"/>
+    <d v="2026-09-06T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0025"/>
+    <s v="Rheinmeal s.r.o."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-09-12T00:00:00"/>
+    <x v="3"/>
+    <n v="6"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0014"/>
+    <d v="2026-10-03T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0006"/>
+    <s v="Vltatronic Sp. z o.o."/>
+    <s v="country"/>
+    <s v="consistency"/>
+    <s v="Country is not a standard English name / ISO code"/>
+    <s v="Map to ISO code PL"/>
+    <s v="Medium"/>
+    <s v="In Progress"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0015"/>
+    <d v="2026-09-07T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0060"/>
+    <s v="KRAFTFORM SAS"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="In Progress"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="4"/>
+    <n v="28"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0016"/>
+    <d v="2026-09-25T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0056"/>
+    <s v="Teraplast GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="2"/>
+    <n v="10"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0017"/>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0012"/>
+    <s v="Boracast GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="3"/>
+    <n v="34"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0018"/>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0001"/>
+    <s v="FERROMETAL GMBH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="In Progress"/>
+    <s v="S. Kaya"/>
+    <m/>
+    <x v="1"/>
+    <n v="4"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0019"/>
+    <d v="2026-09-27T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0008"/>
+    <s v="KRAFTGUSS S.R.O."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="0"/>
+    <n v="8"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0020"/>
+    <d v="2026-09-18T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0005"/>
+    <s v="Ferrocast  GmbH"/>
+    <s v="country"/>
+    <s v="consistency"/>
+    <s v="Country is not a standard English name / ISO code"/>
+    <s v="Map to ISO code DE"/>
+    <s v="Medium"/>
+    <s v="In Progress"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="4"/>
+    <n v="17"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0021"/>
+    <d v="2026-09-22T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0039"/>
+    <s v="Atlastronc GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="S. Kaya"/>
+    <m/>
+    <x v="3"/>
+    <n v="13"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0022"/>
+    <d v="2026-09-08T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0040"/>
+    <s v="Ventoguss"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="27"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0023"/>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0058"/>
+    <s v="Deltaflex  Sp.  z  o.o."/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="S. Kaya"/>
+    <m/>
+    <x v="2"/>
+    <n v="34"/>
+    <n v="20"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0024"/>
+    <d v="2026-09-12T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0024"/>
+    <s v="Velacast  GmbH"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-09-16T00:00:00"/>
+    <x v="1"/>
+    <n v="4"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0025"/>
+    <d v="2026-10-03T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0069"/>
+    <s v="Kraftflex"/>
+    <s v="vat_number"/>
+    <s v="consistency"/>
+    <s v="VAT ID contains spaces"/>
+    <s v="Remove spaces during migration"/>
+    <s v="Low"/>
+    <s v="Open"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="0"/>
+    <n v="2"/>
+    <n v="20"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0026"/>
+    <d v="2026-09-27T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100055"/>
+    <s v="Deltaplast GmbH"/>
+    <s v="terms"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'terms' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-09-29T00:00:00"/>
+    <x v="3"/>
+    <n v="2"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0027"/>
+    <d v="2026-09-27T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100186"/>
+    <s v="Alpentronic GmbH"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="M. Chen"/>
+    <d v="2026-09-28T00:00:00"/>
+    <x v="1"/>
+    <n v="1"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0028"/>
+    <d v="2026-09-20T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100334"/>
+    <s v="Lumencast GmbH"/>
+    <s v="iban"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'iban' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="4"/>
+    <n v="1"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0029"/>
+    <d v="2026-09-12T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100334"/>
+    <s v="Lumencast GmbH"/>
+    <s v="terms"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'terms' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="In Progress"/>
+    <s v="J. Novak"/>
+    <m/>
+    <x v="4"/>
+    <n v="23"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0030"/>
+    <d v="2026-09-07T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100247"/>
+    <s v="Voltaflex GmbH"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="2"/>
+    <n v="28"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0031"/>
+    <d v="2026-09-14T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100168"/>
+    <s v="Kraftseal S.r.l."/>
+    <s v="iban"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'iban' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="In Progress"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="1"/>
+    <n v="21"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0032"/>
+    <d v="2026-09-22T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100216"/>
+    <s v="Alpenwerk GmbH"/>
+    <s v="terms"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'terms' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Closed"/>
+    <s v="A. Weber"/>
+    <d v="2026-09-29T00:00:00"/>
+    <x v="4"/>
+    <n v="7"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0033"/>
+    <d v="2026-09-05T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100367"/>
+    <s v="Ferroparts GmbH"/>
+    <s v="vat"/>
+    <s v="validity"/>
+    <s v="VAT ID does not match the DE format"/>
+    <s v="Verify VAT ID (e.g. EU VIES check)"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="J. Novak"/>
+    <m/>
+    <x v="1"/>
+    <n v="30"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0034"/>
+    <d v="2026-09-16T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100153"/>
+    <s v="Atlasplast Sp. z o.o."/>
+    <s v="vat"/>
+    <s v="validity"/>
+    <s v="VAT ID does not match the PL format"/>
+    <s v="Verify VAT ID (e.g. EU VIES check)"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="1"/>
+    <n v="19"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0035"/>
+    <d v="2026-09-24T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100162"/>
+    <s v="Tauroform Sp. z o.o."/>
+    <s v="iban"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'iban' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Waiting"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="0"/>
+    <n v="11"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0036"/>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100071"/>
+    <s v="Cerrowerk Sp. z o.o."/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-10-04T00:00:00"/>
+    <x v="2"/>
+    <n v="3"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0037"/>
+    <d v="2026-09-12T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100011"/>
+    <s v="Novaform GmbH"/>
+    <s v="iban"/>
+    <s v="validity"/>
+    <s v="IBAN fails length or check-digit test"/>
+    <s v="Block payments until bank data is confirmed"/>
+    <s v="High"/>
+    <s v="Waiting"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="4"/>
+    <n v="23"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0038"/>
+    <d v="2026-09-15T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100387"/>
+    <s v="Lumenparts GmbH"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-09-19T00:00:00"/>
+    <x v="3"/>
+    <n v="4"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0039"/>
+    <d v="2026-09-11T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100019"/>
+    <s v="Ferrocast GmbH"/>
+    <s v="iban"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'iban' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="L. Rossi"/>
+    <d v="2026-09-20T00:00:00"/>
+    <x v="4"/>
+    <n v="9"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0040"/>
+    <d v="2026-09-25T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100314"/>
+    <s v="Voltaplast GmbH"/>
+    <s v="terms"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'terms' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Closed"/>
+    <s v="A. Weber"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="2"/>
+    <n v="10"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0041"/>
+    <d v="2026-09-27T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100302"/>
+    <s v="Boraline GmbH"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="8"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0042"/>
+    <d v="2026-09-03T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100127"/>
+    <s v="Rheinplast S.r.l."/>
+    <s v="terms"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'terms' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="In Progress"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="3"/>
+    <n v="32"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0043"/>
+    <d v="2026-09-16T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100007"/>
+    <s v="Terraparts GmbH"/>
+    <s v="vat"/>
+    <s v="validity"/>
+    <s v="VAT ID does not match the DE format"/>
+    <s v="Verify VAT ID (e.g. EU VIES check)"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="M. Chen"/>
+    <d v="2026-09-23T00:00:00"/>
+    <x v="2"/>
+    <n v="7"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0044"/>
+    <d v="2026-09-27T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100224"/>
+    <s v="Ventometal GmbH"/>
+    <s v="iban"/>
+    <s v="validity"/>
+    <s v="IBAN fails length or check-digit test"/>
+    <s v="Block payments until bank data is confirmed"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="S. Kaya"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="3"/>
+    <n v="8"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0045"/>
+    <d v="2026-09-19T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100030"/>
+    <s v="Nordwerk GmbH"/>
+    <s v="vat"/>
+    <s v="validity"/>
+    <s v="VAT ID does not match the AT format"/>
+    <s v="Verify VAT ID (e.g. EU VIES check)"/>
+    <s v="High"/>
+    <s v="In Progress"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="4"/>
+    <n v="16"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0046"/>
+    <d v="2026-09-09T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100132"/>
+    <s v="Silberwerk s.r.o."/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="J. Novak"/>
+    <m/>
+    <x v="2"/>
+    <n v="26"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0047"/>
+    <d v="2026-09-05T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0023"/>
+    <s v="Cerroline GmbH"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="In Progress"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="2"/>
+    <n v="30"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0048"/>
+    <d v="2026-09-02T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0042"/>
+    <s v="Voltawerk"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="S. Kaya"/>
+    <m/>
+    <x v="0"/>
+    <n v="33"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0049"/>
+    <d v="2026-09-29T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0054"/>
+    <s v="Boralne GmbH"/>
+    <s v="postcode"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'postcode' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="6"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0050"/>
+    <d v="2026-09-12T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0041"/>
+    <s v="Cerroparts"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="In Progress"/>
+    <s v="J. Novak"/>
+    <m/>
+    <x v="1"/>
+    <n v="23"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0051"/>
+    <d v="2026-09-09T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0041"/>
+    <s v="Cerroparts"/>
+    <s v="postcode"/>
+    <s v="validity"/>
+    <s v="Postcode length is wrong for DE"/>
+    <s v="Correct postcode"/>
+    <s v="Medium"/>
+    <s v="Open"/>
+    <s v="L. Rossi"/>
+    <m/>
+    <x v="1"/>
+    <n v="26"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0052"/>
+    <d v="2026-09-29T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0044"/>
+    <s v="Novasel GmbH"/>
+    <s v="postcode"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'postcode' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Closed"/>
+    <s v="J. Novak"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="4"/>
+    <n v="6"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0053"/>
+    <d v="2026-09-09T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0061"/>
+    <s v="Boraetal Sp. z o.o."/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Waiting"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="3"/>
+    <n v="26"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0054"/>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0030"/>
+    <s v="Kraftcast  Sp.  z  o.o."/>
+    <s v="postcode"/>
+    <s v="validity"/>
+    <s v="Postcode length is wrong for PL"/>
+    <s v="Correct postcode"/>
+    <s v="Medium"/>
+    <s v="Closed"/>
+    <s v="A. Weber"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="1"/>
+    <n v="4"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0055"/>
+    <d v="2026-09-02T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0025"/>
+    <s v="Rheinmeal s.r.o."/>
+    <s v="postcode"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'postcode' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="Medium"/>
+    <s v="Waiting"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="3"/>
+    <n v="33"/>
+    <n v="10"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0056"/>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="ERP_B"/>
+    <s v="SUP-0020"/>
+    <s v="Polarmetal"/>
+    <s v="vat"/>
+    <s v="completeness"/>
+    <s v="Mandatory field 'vat' is empty"/>
+    <s v="Request value from supplier / purchasing"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="4"/>
+    <n v="4"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0057"/>
+    <d v="2026-09-21T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100234"/>
+    <s v="Nordcast Sp. z o.o."/>
+    <s v="record"/>
+    <s v="uniqueness"/>
+    <s v="Possible duplicate of 0000100417 (Same VAT ID)"/>
+    <s v="Merge into one record before migration"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="A. Weber"/>
+    <m/>
+    <x v="0"/>
+    <n v="14"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0058"/>
+    <d v="2026-09-05T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100238"/>
+    <s v="Primaform S.r.l."/>
+    <s v="record"/>
+    <s v="uniqueness"/>
+    <s v="Possible duplicate of 0000100422 (Same VAT ID)"/>
+    <s v="Merge into one record before migration"/>
+    <s v="High"/>
+    <s v="In Progress"/>
+    <s v="M. Chen"/>
+    <m/>
+    <x v="1"/>
+    <n v="30"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <s v="T-0059"/>
+    <d v="2026-09-03T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100177"/>
+    <s v="Atlasguss GmbH"/>
+    <s v="record"/>
+    <s v="uniqueness"/>
+    <s v="Possible duplicate of 0000100412 (Same VAT ID)"/>
+    <s v="Merge into one record before migration"/>
+    <s v="High"/>
+    <s v="Closed"/>
+    <s v="M. Chen"/>
+    <d v="2026-09-06T00:00:00"/>
+    <x v="3"/>
+    <n v="3"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="T-0060"/>
+    <d v="2026-09-23T00:00:00"/>
+    <s v="ERP_A"/>
+    <s v="0000100418"/>
+    <s v="Lumenform  GmbH"/>
+    <s v="record"/>
+    <s v="uniqueness"/>
+    <s v="Possible duplicate of 0000100192 (Same VAT ID)"/>
+    <s v="Merge into one record before migration"/>
+    <s v="High"/>
+    <s v="Open"/>
+    <s v="S. Kaya"/>
+    <m/>
+    <x v="2"/>
+    <n v="12"/>
+    <n v="5"/>
+    <x v="1"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77F7C93B-80DE-0C41-978F-59480CEB1DAB}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A8:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="13"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="16"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Ticket ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2186,18 +3520,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12509E95-5F09-DC49-B9BC-77DD19A10A22}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>561</v>
       </c>
@@ -2206,7 +3543,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>562</v>
       </c>
@@ -2215,13 +3552,119 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>563</v>
       </c>
       <c r="B5">
         <f ca="1">COUNTIFS(tblTickets[Status],"&lt;&gt;Closed",tblTickets[SLA Status],"Breached")</f>
         <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="B9" t="s">
+        <v>567</v>
+      </c>
+      <c r="C9" t="s">
+        <v>568</v>
+      </c>
+      <c r="D9" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10" s="4">
+        <v>7</v>
+      </c>
+      <c r="C10" s="4">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B11" s="4">
+        <v>6</v>
+      </c>
+      <c r="C11" s="4">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" s="4">
+        <v>6</v>
+      </c>
+      <c r="C12" s="4">
+        <v>5</v>
+      </c>
+      <c r="D12" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="B13" s="4">
+        <v>6</v>
+      </c>
+      <c r="C13" s="4">
+        <v>6</v>
+      </c>
+      <c r="D13" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B14" s="4">
+        <v>7</v>
+      </c>
+      <c r="C14" s="4">
+        <v>5</v>
+      </c>
+      <c r="D14" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="B15" s="4">
+        <v>32</v>
+      </c>
+      <c r="C15" s="4">
+        <v>28</v>
+      </c>
+      <c r="D15" s="4">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel lesson 3 (part 5): Status slicer for the Dashboard PivotTable
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE441EC-A384-0D46-A1BB-2EFD8476A3F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE566B6-5ACF-3B44-8F2B-B29CC09FB0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="520" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,21 @@
   <definedNames>
     <definedName name="lstPriority">Lists!$B$2:$B$4</definedName>
     <definedName name="lstStatus">Lists!$A$2:$A$5</definedName>
+    <definedName name="Slicer_Status">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId6"/>
+    <pivotCache cacheId="5" r:id="rId6"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId7"/>
+      </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -1892,6 +1901,89 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>142869</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Status">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3E8B6AD-1135-8712-C1E0-141103FA0990}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Status"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4254500" y="1333500"/>
+              <a:ext cx="1828800" cy="2428869"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="mac" refreshedDate="46300.604069444445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="60" xr:uid="{E198A4B9-9466-014B-B142-729ED828A4DF}">
   <cacheSource type="worksheet">
@@ -1929,7 +2021,12 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="Status" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="4">
+        <s v="Closed"/>
+        <s v="In Progress"/>
+        <s v="Open"/>
+        <s v="Waiting"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Owner" numFmtId="0">
       <sharedItems/>
@@ -1961,7 +2058,7 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
+      <x14:pivotCacheDefinition pivotCacheId="1181872588"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -1980,7 +2077,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="0"/>
@@ -1999,7 +2096,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="1"/>
@@ -2018,7 +2115,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="J. Novak"/>
     <m/>
     <x v="0"/>
@@ -2037,7 +2134,7 @@
     <s v="Country is not a standard English name / ISO code"/>
     <s v="Map to ISO code DE"/>
     <s v="Medium"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="M. Chen"/>
     <m/>
     <x v="0"/>
@@ -2056,7 +2153,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2075,7 +2172,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="2"/>
@@ -2094,7 +2191,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="A. Weber"/>
     <d v="2026-09-03T00:00:00"/>
     <x v="2"/>
@@ -2113,7 +2210,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="3"/>
@@ -2132,7 +2229,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-09-08T00:00:00"/>
     <x v="4"/>
@@ -2151,7 +2248,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="M. Chen"/>
     <m/>
     <x v="1"/>
@@ -2170,7 +2267,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2189,7 +2286,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="J. Novak"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="3"/>
@@ -2208,7 +2305,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-09-12T00:00:00"/>
     <x v="3"/>
@@ -2227,7 +2324,7 @@
     <s v="Country is not a standard English name / ISO code"/>
     <s v="Map to ISO code PL"/>
     <s v="Medium"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2246,7 +2343,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="M. Chen"/>
     <m/>
     <x v="4"/>
@@ -2265,7 +2362,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="2"/>
@@ -2284,7 +2381,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="3"/>
@@ -2303,7 +2400,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="S. Kaya"/>
     <m/>
     <x v="1"/>
@@ -2322,7 +2419,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="0"/>
@@ -2341,7 +2438,7 @@
     <s v="Country is not a standard English name / ISO code"/>
     <s v="Map to ISO code DE"/>
     <s v="Medium"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="M. Chen"/>
     <m/>
     <x v="4"/>
@@ -2360,7 +2457,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="S. Kaya"/>
     <m/>
     <x v="3"/>
@@ -2379,7 +2476,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2398,7 +2495,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="S. Kaya"/>
     <m/>
     <x v="2"/>
@@ -2417,7 +2514,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-09-16T00:00:00"/>
     <x v="1"/>
@@ -2436,7 +2533,7 @@
     <s v="VAT ID contains spaces"/>
     <s v="Remove spaces during migration"/>
     <s v="Low"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="0"/>
@@ -2455,7 +2552,7 @@
     <s v="Mandatory field 'terms' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-09-29T00:00:00"/>
     <x v="3"/>
@@ -2474,7 +2571,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="M. Chen"/>
     <d v="2026-09-28T00:00:00"/>
     <x v="1"/>
@@ -2493,7 +2590,7 @@
     <s v="Mandatory field 'iban' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-09-21T00:00:00"/>
     <x v="4"/>
@@ -2512,7 +2609,7 @@
     <s v="Mandatory field 'terms' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="J. Novak"/>
     <m/>
     <x v="4"/>
@@ -2531,7 +2628,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="2"/>
@@ -2550,7 +2647,7 @@
     <s v="Mandatory field 'iban' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="A. Weber"/>
     <m/>
     <x v="1"/>
@@ -2569,7 +2666,7 @@
     <s v="Mandatory field 'terms' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="A. Weber"/>
     <d v="2026-09-29T00:00:00"/>
     <x v="4"/>
@@ -2588,7 +2685,7 @@
     <s v="VAT ID does not match the DE format"/>
     <s v="Verify VAT ID (e.g. EU VIES check)"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="J. Novak"/>
     <m/>
     <x v="1"/>
@@ -2607,7 +2704,7 @@
     <s v="VAT ID does not match the PL format"/>
     <s v="Verify VAT ID (e.g. EU VIES check)"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="M. Chen"/>
     <m/>
     <x v="1"/>
@@ -2626,7 +2723,7 @@
     <s v="Mandatory field 'iban' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Waiting"/>
+    <x v="3"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="0"/>
@@ -2645,7 +2742,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-10-04T00:00:00"/>
     <x v="2"/>
@@ -2664,7 +2761,7 @@
     <s v="IBAN fails length or check-digit test"/>
     <s v="Block payments until bank data is confirmed"/>
     <s v="High"/>
-    <s v="Waiting"/>
+    <x v="3"/>
     <s v="M. Chen"/>
     <m/>
     <x v="4"/>
@@ -2683,7 +2780,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-09-19T00:00:00"/>
     <x v="3"/>
@@ -2702,7 +2799,7 @@
     <s v="Mandatory field 'iban' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="L. Rossi"/>
     <d v="2026-09-20T00:00:00"/>
     <x v="4"/>
@@ -2721,7 +2818,7 @@
     <s v="Mandatory field 'terms' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="A. Weber"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="2"/>
@@ -2740,7 +2837,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2759,7 +2856,7 @@
     <s v="Mandatory field 'terms' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="M. Chen"/>
     <m/>
     <x v="3"/>
@@ -2778,7 +2875,7 @@
     <s v="VAT ID does not match the DE format"/>
     <s v="Verify VAT ID (e.g. EU VIES check)"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="M. Chen"/>
     <d v="2026-09-23T00:00:00"/>
     <x v="2"/>
@@ -2797,7 +2894,7 @@
     <s v="IBAN fails length or check-digit test"/>
     <s v="Block payments until bank data is confirmed"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="S. Kaya"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="3"/>
@@ -2816,7 +2913,7 @@
     <s v="VAT ID does not match the AT format"/>
     <s v="Verify VAT ID (e.g. EU VIES check)"/>
     <s v="High"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="A. Weber"/>
     <m/>
     <x v="4"/>
@@ -2835,7 +2932,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="J. Novak"/>
     <m/>
     <x v="2"/>
@@ -2854,7 +2951,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="2"/>
@@ -2873,7 +2970,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="S. Kaya"/>
     <m/>
     <x v="0"/>
@@ -2892,7 +2989,7 @@
     <s v="Mandatory field 'postcode' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -2911,7 +3008,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="J. Novak"/>
     <m/>
     <x v="1"/>
@@ -2930,7 +3027,7 @@
     <s v="Postcode length is wrong for DE"/>
     <s v="Correct postcode"/>
     <s v="Medium"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="L. Rossi"/>
     <m/>
     <x v="1"/>
@@ -2949,7 +3046,7 @@
     <s v="Mandatory field 'postcode' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="J. Novak"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="4"/>
@@ -2968,7 +3065,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Waiting"/>
+    <x v="3"/>
     <s v="A. Weber"/>
     <m/>
     <x v="3"/>
@@ -2987,7 +3084,7 @@
     <s v="Postcode length is wrong for PL"/>
     <s v="Correct postcode"/>
     <s v="Medium"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="A. Weber"/>
     <d v="2026-10-05T00:00:00"/>
     <x v="1"/>
@@ -3006,7 +3103,7 @@
     <s v="Mandatory field 'postcode' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="Medium"/>
-    <s v="Waiting"/>
+    <x v="3"/>
     <s v="A. Weber"/>
     <m/>
     <x v="3"/>
@@ -3025,7 +3122,7 @@
     <s v="Mandatory field 'vat' is empty"/>
     <s v="Request value from supplier / purchasing"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="M. Chen"/>
     <m/>
     <x v="4"/>
@@ -3044,7 +3141,7 @@
     <s v="Possible duplicate of 0000100417 (Same VAT ID)"/>
     <s v="Merge into one record before migration"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="A. Weber"/>
     <m/>
     <x v="0"/>
@@ -3063,7 +3160,7 @@
     <s v="Possible duplicate of 0000100422 (Same VAT ID)"/>
     <s v="Merge into one record before migration"/>
     <s v="High"/>
-    <s v="In Progress"/>
+    <x v="1"/>
     <s v="M. Chen"/>
     <m/>
     <x v="1"/>
@@ -3082,7 +3179,7 @@
     <s v="Possible duplicate of 0000100412 (Same VAT ID)"/>
     <s v="Merge into one record before migration"/>
     <s v="High"/>
-    <s v="Closed"/>
+    <x v="0"/>
     <s v="M. Chen"/>
     <d v="2026-09-06T00:00:00"/>
     <x v="3"/>
@@ -3101,7 +3198,7 @@
     <s v="Possible duplicate of 0000100192 (Same VAT ID)"/>
     <s v="Merge into one record before migration"/>
     <s v="High"/>
-    <s v="Open"/>
+    <x v="2"/>
     <s v="S. Kaya"/>
     <m/>
     <x v="2"/>
@@ -3113,7 +3210,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77F7C93B-80DE-0C41-978F-59480CEB1DAB}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77F7C93B-80DE-0C41-978F-59480CEB1DAB}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A8:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -3126,7 +3223,15 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -3199,6 +3304,30 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Status" xr10:uid="{E21674C6-27D6-B845-917A-2DDD4FEB2A03}" sourceName="Status">
+  <pivotTables>
+    <pivotTable tabId="5" name="PivotTable1"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1181872588">
+      <items count="4">
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
+        <i x="2" s="1"/>
+        <i x="3" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Status" xr10:uid="{D1423163-F858-A643-B06C-80588E382D3E}" cache="Slicer_Status" caption="Status" rowHeight="230716"/>
+</slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3669,6 +3798,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId3"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Excel lesson 3 (part 6): slicer set to open tickets (Open, In Progress, Waiting)
</commit_message>
<xml_diff>
--- a/excel/BU2_Ticket_Tracker.xlsx
+++ b/excel/BU2_Ticket_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE566B6-5ACF-3B44-8F2B-B29CC09FB0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD6C5201-5C3D-E84D-BF31-DA9A66C73D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="520" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3225,7 +3225,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="5">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
@@ -3314,7 +3314,7 @@
   <data>
     <tabular pivotCacheId="1181872588">
       <items count="4">
-        <i x="0" s="1"/>
+        <i x="0"/>
         <i x="1" s="1"/>
         <i x="2" s="1"/>
         <i x="3" s="1"/>
@@ -3720,10 +3720,10 @@
         <v>7</v>
       </c>
       <c r="C10" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D10" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -3731,13 +3731,13 @@
         <v>250</v>
       </c>
       <c r="B11" s="4">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4">
         <v>6</v>
-      </c>
-      <c r="C11" s="4">
-        <v>5</v>
-      </c>
-      <c r="D11" s="4">
-        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -3745,13 +3745,13 @@
         <v>285</v>
       </c>
       <c r="B12" s="4">
+        <v>5</v>
+      </c>
+      <c r="C12" s="4">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4">
         <v>6</v>
-      </c>
-      <c r="C12" s="4">
-        <v>5</v>
-      </c>
-      <c r="D12" s="4">
-        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -3759,13 +3759,13 @@
         <v>241</v>
       </c>
       <c r="B13" s="4">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4">
         <v>6</v>
-      </c>
-      <c r="C13" s="4">
-        <v>6</v>
-      </c>
-      <c r="D13" s="4">
-        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -3776,10 +3776,10 @@
         <v>7</v>
       </c>
       <c r="C14" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D14" s="4">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -3787,13 +3787,13 @@
         <v>565</v>
       </c>
       <c r="B15" s="4">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C15" s="4">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D15" s="4">
-        <v>60</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>